<commit_message>
Refresh capability model and publication date
</commit_message>
<xml_diff>
--- a/public/reports/personal-ai-four-year-capability-report-card.xlsx
+++ b/public/reports/personal-ai-four-year-capability-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rff52c49673124acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report Card" sheetId="2" r:id="R54ce1de8f7dc4f7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="3" r:id="Re6fa9bf3a6b4475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="4" r:id="R2e6b8911a2884d1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="5" r:id="R2c6234a01d8e49d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" r:id="R33a286edf86b4704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2cd0f9f4e14a499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report Card" sheetId="2" r:id="R1ff0822245974b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="3" r:id="R50d4464d4cee4fec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="4" r:id="Raa0e665def6f4808"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="5" r:id="R8b1f9d2dd0f04d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" r:id="R719f51eba8a84489"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,13 +18,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="0.000"/>
     <x:numFmt numFmtId="204" formatCode="0.0"/>
-    <x:numFmt numFmtId="205" formatCode="0.00"/>
+    <x:numFmt numFmtId="205" formatCode="+0.000;-0.000;0.000"/>
+    <x:numFmt numFmtId="206" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="8">
     <x:font>
@@ -140,7 +141,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="61">
+  <x:cellXfs count="64">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -257,10 +258,10 @@
     <x:xf numFmtId="0" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="205" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -272,10 +273,19 @@
     <x:xf numFmtId="202" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="206" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="206" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="205" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -588,7 +598,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -610,7 +620,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rff94b147f4cd460d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd21268bed9ce48ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -620,7 +630,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BenchmarkObservationsTable" displayName="BenchmarkObservationsTable" ref="A5:K41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BenchmarkObservationsTable" displayName="BenchmarkObservationsTable" ref="A5:K45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Benchmark ID"/>
     <x:tableColumn id="2" name="Benchmark Name"/>
@@ -671,9 +681,9 @@
     <x:tableColumn id="11" name="Prior-2 depth"/>
     <x:tableColumn id="12" name="Prior depth"/>
     <x:tableColumn id="13" name="Latest depth"/>
-    <x:tableColumn id="14" name="Recent velocity"/>
-    <x:tableColumn id="15" name="Prior velocity"/>
-    <x:tableColumn id="16" name="Acceleration"/>
+    <x:tableColumn id="14" name="Recent gap velocity"/>
+    <x:tableColumn id="15" name="Prior gap velocity"/>
+    <x:tableColumn id="16" name="Gap acceleration"/>
     <x:tableColumn id="17" name="Projection basis"/>
     <x:tableColumn id="18" name="Current score"/>
     <x:tableColumn id="19" name="Letter"/>
@@ -884,11 +894,11 @@
     <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="3" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="13" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="13" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
@@ -1039,71 +1049,71 @@
     <x:row r="4"/>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="9" t="str">
-        <x:v>OVERALL GPA</x:v>
+        <x:v>CURRENT SCORE</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>OVERALL GPA</x:v>
+        <x:v>CURRENT SCORE</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>OVERALL GPA</x:v>
+        <x:v>CURRENT SCORE</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>CURRENT SCORE</x:v>
+        <x:v>CURRENT LETTER</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>CURRENT SCORE</x:v>
+        <x:v>CURRENT LETTER</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>CURRENT SCORE</x:v>
-      </x:c>
-      <x:c r="G5" s="9" t="str">
-        <x:v>GRADED COVERAGE</x:v>
-      </x:c>
-      <x:c r="H5" s="9" t="str">
-        <x:v>GRADED COVERAGE</x:v>
-      </x:c>
-      <x:c r="I5" s="9" t="str">
-        <x:v>GRADED COVERAGE</x:v>
-      </x:c>
-      <x:c r="J5" s="48" t="str">
+        <x:v>CURRENT LETTER</x:v>
+      </x:c>
+      <x:c r="G5" s="48" t="str">
         <x:v>2028-Q4 SCORE</x:v>
       </x:c>
-      <x:c r="K5" s="48" t="str">
+      <x:c r="H5" s="48" t="str">
         <x:v>2028-Q4 SCORE</x:v>
       </x:c>
-      <x:c r="L5" s="48" t="str">
+      <x:c r="I5" s="48" t="str">
         <x:v>2028-Q4 SCORE</x:v>
       </x:c>
+      <x:c r="J5" s="9" t="str">
+        <x:v>GAP ACCELERATION / QTR²</x:v>
+      </x:c>
+      <x:c r="K5" s="9" t="str">
+        <x:v>GAP ACCELERATION / QTR²</x:v>
+      </x:c>
+      <x:c r="L5" s="9" t="str">
+        <x:v>GAP ACCELERATION / QTR²</x:v>
+      </x:c>
       <x:c r="M5" s="9" t="str">
-        <x:v>CURRENT LETTER</x:v>
+        <x:v>ACCELERATION COVERAGE</x:v>
       </x:c>
       <x:c r="N5" s="9" t="str">
-        <x:v>CURRENT LETTER</x:v>
+        <x:v>ACCELERATION COVERAGE</x:v>
       </x:c>
       <x:c r="O5" s="9" t="str">
-        <x:v>CURRENT LETTER</x:v>
+        <x:v>ACCELERATION COVERAGE</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="54" t="n">
-        <x:f>AVERAGE('Summary'!$E$13:$E$16)</x:f>
-        <x:v>0.6696428571428572</x:v>
-      </x:c>
-      <x:c r="D6" s="55" t="n">
         <x:f>AVERAGE('Summary'!$D$13:$D$16)</x:f>
-        <x:v>0.4461357386309524</x:v>
-      </x:c>
-      <x:c r="G6" s="56" t="n">
-        <x:f>COUNTIF('Report Card'!$AT$6:$AT$28,"&lt;&gt;N/A")/ROWS('Report Card'!$AT$6:$AT$28)</x:f>
-        <x:v>0.6956521739130435</x:v>
+        <x:v>0.4666192850127242</x:v>
+      </x:c>
+      <x:c r="D6" s="53" t="str">
+        <x:f>IF(A6&gt;='Methodology'!$G$7,"A",IF(A6&gt;='Methodology'!$G$8,"B",IF(A6&gt;='Methodology'!$G$9,"C",IF(A6&gt;='Methodology'!$G$10,"D","F"))))</x:f>
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G6" s="54" t="n">
+        <x:f>AVERAGE('Summary'!$F$13:$F$16)</x:f>
+        <x:v>0.6420458316228199</x:v>
       </x:c>
       <x:c r="J6" s="55" t="n">
-        <x:f>AVERAGE('Summary'!$F$13:$F$16)</x:f>
-        <x:v>0.6233766173378316</x:v>
-      </x:c>
-      <x:c r="M6" s="53" t="str">
-        <x:f>IF(D6&gt;='Methodology'!$G$7,"A",IF(D6&gt;='Methodology'!$G$8,"B",IF(D6&gt;='Methodology'!$G$9,"C",IF(D6&gt;='Methodology'!$G$10,"D","F"))))</x:f>
-        <x:v>F</x:v>
+        <x:f>IFERROR(AVERAGE('Summary'!$H$13:$H$16),"")</x:f>
+        <x:v>0.05795221995259677</x:v>
+      </x:c>
+      <x:c r="M6" s="56" t="n">
+        <x:f>COUNTIF('Model'!$D$6:$D$28,"&gt;=3")/COUNTIF('Model'!$D$6:$D$28,"&gt;0")</x:f>
+        <x:v>0.3</x:v>
       </x:c>
     </x:row>
     <x:row r="7"/>
@@ -1129,6 +1139,15 @@
       <x:c r="F11" s="9" t="str">
         <x:v>CATEGORY REPORT CARD</x:v>
       </x:c>
+      <x:c r="G11" s="9" t="str">
+        <x:v>CATEGORY REPORT CARD</x:v>
+      </x:c>
+      <x:c r="H11" s="9" t="str">
+        <x:v>CATEGORY REPORT CARD</x:v>
+      </x:c>
+      <x:c r="I11" s="9" t="str">
+        <x:v>CATEGORY REPORT CARD</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="13" t="str">
@@ -1149,6 +1168,15 @@
       <x:c r="F12" s="13" t="str">
         <x:v>2028-Q4 score</x:v>
       </x:c>
+      <x:c r="G12" s="13" t="str">
+        <x:v>Gap velocity / qtr</x:v>
+      </x:c>
+      <x:c r="H12" s="13" t="str">
+        <x:v>Gap acceleration / qtr²</x:v>
+      </x:c>
+      <x:c r="I12" s="13" t="str">
+        <x:v>Accel. coverage</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="17" t="str">
@@ -1156,7 +1184,7 @@
       </x:c>
       <x:c r="B13" s="17" t="n">
         <x:f>COUNTIFS('Report Card'!$A$6:$A$28,A13,'Report Card'!$AT$6:$AT$28,"&lt;&gt;N/A")</x:f>
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C13" s="17" t="n">
         <x:f>COUNTIF('Report Card'!$A$6:$A$28,A13)</x:f>
@@ -1164,7 +1192,7 @@
       </x:c>
       <x:c r="D13" s="24" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,A13,'Report Card'!$AS$6:$AS$28),"")</x:f>
-        <x:v>0.32918581166666666</x:v>
+        <x:v>0.411119997193754</x:v>
       </x:c>
       <x:c r="E13" s="59" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,A13,'Report Card'!$AU$6:$AU$28),"")</x:f>
@@ -1172,7 +1200,19 @@
       </x:c>
       <x:c r="F13" s="24" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,A13,'Report Card'!$AQ$6:$AQ$28),"")</x:f>
-        <x:v>0.34188613611131996</x:v>
+        <x:v>0.41656299325127366</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$N$6:$N$28,'Model'!$C$6:$C$28,A13,'Model'!$D$6:$D$28,"&gt;=2"),"")</x:f>
+        <x:v>0.006549844650824333</x:v>
+      </x:c>
+      <x:c r="H13" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$P$6:$P$28,'Model'!$C$6:$C$28,A13,'Model'!$D$6:$D$28,"&gt;=3"),"")</x:f>
+        <x:v>-0.0718969048742778</x:v>
+      </x:c>
+      <x:c r="I13" s="19" t="n">
+        <x:f>IFERROR(COUNTIFS('Model'!$C$6:$C$28,A13,'Model'!$D$6:$D$28,"&gt;=3")/COUNTIFS('Model'!$C$6:$C$28,A13,'Model'!$D$6:$D$28,"&gt;0"),"")</x:f>
+        <x:v>0.14285714285714285</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1199,6 +1239,18 @@
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,A14,'Report Card'!$AQ$6:$AQ$28),"")</x:f>
         <x:v>0.7614002449377768</x:v>
       </x:c>
+      <x:c r="G14" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$N$6:$N$28,'Model'!$C$6:$C$28,A14,'Model'!$D$6:$D$28,"&gt;=2"),"")</x:f>
+        <x:v>0.21231534925022855</x:v>
+      </x:c>
+      <x:c r="H14" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$P$6:$P$28,'Model'!$C$6:$C$28,A14,'Model'!$D$6:$D$28,"&gt;=3"),"")</x:f>
+        <x:v>0.06540560141180742</x:v>
+      </x:c>
+      <x:c r="I14" s="19" t="n">
+        <x:f>IFERROR(COUNTIFS('Model'!$C$6:$C$28,A14,'Model'!$D$6:$D$28,"&gt;=3")/COUNTIFS('Model'!$C$6:$C$28,A14,'Model'!$D$6:$D$28,"&gt;0"),"")</x:f>
+        <x:v>0.5714285714285714</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="17" t="str">
@@ -1224,6 +1276,17 @@
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,A15,'Report Card'!$AQ$6:$AQ$28),"")</x:f>
         <x:v>0.5390515200198509</x:v>
       </x:c>
+      <x:c r="G15" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$N$6:$N$28,'Model'!$C$6:$C$28,A15,'Model'!$D$6:$D$28,"&gt;=2"),"")</x:f>
+        <x:v>0.060208192614823824</x:v>
+      </x:c>
+      <x:c r="H15" s="61" t="str">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$P$6:$P$28,'Model'!$C$6:$C$28,A15,'Model'!$D$6:$D$28,"&gt;=3"),"")</x:f>
+      </x:c>
+      <x:c r="I15" s="19" t="n">
+        <x:f>IFERROR(COUNTIFS('Model'!$C$6:$C$28,A15,'Model'!$D$6:$D$28,"&gt;=3")/COUNTIFS('Model'!$C$6:$C$28,A15,'Model'!$D$6:$D$28,"&gt;0"),"")</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
@@ -1249,6 +1312,18 @@
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,A16,'Report Card'!$AQ$6:$AQ$28),"")</x:f>
         <x:v>0.8511685682823786</x:v>
       </x:c>
+      <x:c r="G16" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$N$6:$N$28,'Model'!$C$6:$C$28,A16,'Model'!$D$6:$D$28,"&gt;=2"),"")</x:f>
+        <x:v>0.18665713536174539</x:v>
+      </x:c>
+      <x:c r="H16" s="61" t="n">
+        <x:f>IFERROR(AVERAGEIFS('Model'!$P$6:$P$28,'Model'!$C$6:$C$28,A16,'Model'!$D$6:$D$28,"&gt;=3"),"")</x:f>
+        <x:v>0.18034796332026068</x:v>
+      </x:c>
+      <x:c r="I16" s="19" t="n">
+        <x:f>IFERROR(COUNTIFS('Model'!$C$6:$C$28,A16,'Model'!$D$6:$D$28,"&gt;=3")/COUNTIFS('Model'!$C$6:$C$28,A16,'Model'!$D$6:$D$28,"&gt;0"),"")</x:f>
+        <x:v>0.5</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="57" t="str">
@@ -1256,7 +1331,7 @@
       </x:c>
       <x:c r="B17" s="57" t="n">
         <x:f>SUM(B13:B16)</x:f>
-        <x:v>16</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C17" s="57" t="n">
         <x:f>SUM(C13:C16)</x:f>
@@ -1264,7 +1339,7 @@
       </x:c>
       <x:c r="D17" s="58" t="n">
         <x:f>AVERAGE(D13:D16)</x:f>
-        <x:v>0.4461357386309524</x:v>
+        <x:v>0.4666192850127242</x:v>
       </x:c>
       <x:c r="E17" s="60" t="n">
         <x:f>AVERAGE(E13:E16)</x:f>
@@ -1272,7 +1347,19 @@
       </x:c>
       <x:c r="F17" s="58" t="n">
         <x:f>AVERAGE(F13:F16)</x:f>
-        <x:v>0.6233766173378316</x:v>
+        <x:v>0.6420458316228199</x:v>
+      </x:c>
+      <x:c r="G17" s="62" t="n">
+        <x:f>IFERROR(AVERAGE(G13:G16),"")</x:f>
+        <x:v>0.11643263046940552</x:v>
+      </x:c>
+      <x:c r="H17" s="62" t="n">
+        <x:f>IFERROR(AVERAGE(H13:H16),"")</x:f>
+        <x:v>0.05795221995259677</x:v>
+      </x:c>
+      <x:c r="I17" s="63" t="n">
+        <x:f>COUNTIF('Model'!$D$6:$D$28,"&gt;=3")/COUNTIF('Model'!$D$6:$D$28,"&gt;0")</x:f>
+        <x:v>0.3</x:v>
       </x:c>
     </x:row>
     <x:row r="18"/>
@@ -1527,7 +1614,7 @@
       </x:c>
       <x:c r="B31" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$W$6:$W$28),"")</x:f>
-        <x:v>0.32644676987493987</x:v>
+        <x:v>0.4948350774062049</x:v>
       </x:c>
       <x:c r="C31" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$W$6:$W$28),"")</x:f>
@@ -1543,7 +1630,7 @@
       </x:c>
       <x:c r="F31" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B31:E31),"")</x:f>
-        <x:v>0.4353331210401636</x:v>
+        <x:v>0.4774301979229798</x:v>
       </x:c>
       <x:c r="H31" s="13" t="str">
         <x:v>LEGEND / READING RULE</x:v>
@@ -1562,7 +1649,7 @@
       </x:c>
       <x:c r="B32" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$Y$6:$Y$28),"")</x:f>
-        <x:v>0.32918581166666666</x:v>
+        <x:v>0.411119997193754</x:v>
       </x:c>
       <x:c r="C32" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$Y$6:$Y$28),"")</x:f>
@@ -1578,7 +1665,7 @@
       </x:c>
       <x:c r="F32" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B32:E32),"")</x:f>
-        <x:v>0.4461357386309524</x:v>
+        <x:v>0.4666192850127242</x:v>
       </x:c>
       <x:c r="H32" s="41" t="str">
         <x:v>Observed</x:v>
@@ -1599,7 +1686,7 @@
       </x:c>
       <x:c r="B33" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AA$6:$AA$28),"")</x:f>
-        <x:v>0.3306216996174711</x:v>
+        <x:v>0.41173537761105267</x:v>
       </x:c>
       <x:c r="C33" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AA$6:$AA$28),"")</x:f>
@@ -1615,7 +1702,7 @@
       </x:c>
       <x:c r="F33" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B33:E33),"")</x:f>
-        <x:v>0.47917512805208723</x:v>
+        <x:v>0.4994535475504826</x:v>
       </x:c>
       <x:c r="H33" s="40" t="str">
         <x:v>Carried</x:v>
@@ -1636,7 +1723,7 @@
       </x:c>
       <x:c r="B34" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AC$6:$AC$28),"")</x:f>
-        <x:v>0.3320513393420423</x:v>
+        <x:v>0.41234808035015463</x:v>
       </x:c>
       <x:c r="C34" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AC$6:$AC$28),"")</x:f>
@@ -1652,7 +1739,7 @@
       </x:c>
       <x:c r="F34" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B34:E34),"")</x:f>
-        <x:v>0.5164408735695576</x:v>
+        <x:v>0.5365150588215857</x:v>
       </x:c>
       <x:c r="H34" s="42" t="str">
         <x:v>Projected</x:v>
@@ -1673,7 +1760,7 @@
       </x:c>
       <x:c r="B35" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AE$6:$AE$28),"")</x:f>
-        <x:v>0.3334747580293618</x:v>
+        <x:v>0.4129581169304344</x:v>
       </x:c>
       <x:c r="C35" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AE$6:$AE$28),"")</x:f>
@@ -1689,13 +1776,13 @@
       </x:c>
       <x:c r="F35" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B35:E35),"")</x:f>
-        <x:v>0.5507819567488488</x:v>
+        <x:v>0.5706527964741169</x:v>
       </x:c>
       <x:c r="H35" s="17" t="str">
-        <x:v>Ungraded</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="I35" s="17" t="str">
-        <x:v>Blank score history means the benchmark lacks a defensible normalized observation.</x:v>
+        <x:v>Quarter-over-quarter percentage-point change in the normalized benchmark score; this is not acceleration.</x:v>
       </x:c>
       <x:c r="J35" s="17"/>
       <x:c r="K35" s="17"/>
@@ -1710,7 +1797,7 @@
       </x:c>
       <x:c r="B36" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AG$6:$AG$28),"")</x:f>
-        <x:v>0.33489198275009907</x:v>
+        <x:v>0.41356549895360756</x:v>
       </x:c>
       <x:c r="C36" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AG$6:$AG$28),"")</x:f>
@@ -1726,13 +1813,13 @@
       </x:c>
       <x:c r="F36" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B36:E36),"")</x:f>
-        <x:v>0.5778927878579861</x:v>
+        <x:v>0.5975611669088633</x:v>
       </x:c>
       <x:c r="H36" s="17" t="str">
-        <x:v>GPA</x:v>
+        <x:v>Gap velocity</x:v>
       </x:c>
       <x:c r="I36" s="17" t="str">
-        <x:v>Overall GPA equally weights the four categories; ungraded rows are excluded.</x:v>
+        <x:v>Failure-gap halvings per quarter, estimated only from benchmarks with at least two observations.</x:v>
       </x:c>
       <x:c r="J36" s="17"/>
       <x:c r="K36" s="17"/>
@@ -1747,7 +1834,7 @@
       </x:c>
       <x:c r="B37" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AI$6:$AI$28),"")</x:f>
-        <x:v>0.3363030404571264</x:v>
+        <x:v>0.414170237970905</x:v>
       </x:c>
       <x:c r="C37" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AI$6:$AI$28),"")</x:f>
@@ -1763,13 +1850,13 @@
       </x:c>
       <x:c r="F37" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B37:E37),"")</x:f>
-        <x:v>0.5965284959506749</x:v>
+        <x:v>0.6159952953291195</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
-        <x:v>Caution</x:v>
+        <x:v>Gap acceleration</x:v>
       </x:c>
       <x:c r="I37" s="17" t="str">
-        <x:v>Sparse series project flat or constant velocity. This is a scenario, not a calibrated probability.</x:v>
+        <x:v>Change in failure-gap velocity per quarter², estimated only from benchmarks with at least three observations. Positive means progress is speeding up.</x:v>
       </x:c>
       <x:c r="J37" s="17"/>
       <x:c r="K37" s="17"/>
@@ -1784,7 +1871,7 @@
       </x:c>
       <x:c r="B38" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AK$6:$AK$28),"")</x:f>
-        <x:v>0.3377079579860314</x:v>
+        <x:v>0.41477234548329284</x:v>
       </x:c>
       <x:c r="C38" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AK$6:$AK$28),"")</x:f>
@@ -1800,16 +1887,28 @@
       </x:c>
       <x:c r="F38" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B38:E38),"")</x:f>
-        <x:v>0.6082503756097872</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="15" hidden="0" customHeight="1">
+        <x:v>0.6275164724841026</x:v>
+      </x:c>
+      <x:c r="H38" s="17" t="str">
+        <x:v>Acceleration coverage</x:v>
+      </x:c>
+      <x:c r="I38" s="17" t="str">
+        <x:v>Benchmarks with a 3+ point acceleration estimate divided by graded benchmarks. Coverage prevents a sparse estimate from looking universal.</x:v>
+      </x:c>
+      <x:c r="J38" s="17"/>
+      <x:c r="K38" s="17"/>
+      <x:c r="L38" s="17"/>
+      <x:c r="M38" s="17"/>
+      <x:c r="N38" s="17"/>
+      <x:c r="O38" s="17"/>
+    </x:row>
+    <x:row r="39" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>2028-Q2</x:v>
       </x:c>
       <x:c r="B39" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AM$6:$AM$28),"")</x:f>
-        <x:v>0.33910676205562734</x:v>
+        <x:v>0.41537183294169105</x:v>
       </x:c>
       <x:c r="C39" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AM$6:$AM$28),"")</x:f>
@@ -1825,8 +1924,20 @@
       </x:c>
       <x:c r="F39" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B39:E39),"")</x:f>
-        <x:v>0.6154168176559769</x:v>
-      </x:c>
+        <x:v>0.6344830853774928</x:v>
+      </x:c>
+      <x:c r="H39" s="17" t="str">
+        <x:v>Direct stewardship</x:v>
+      </x:c>
+      <x:c r="I39" s="17" t="str">
+        <x:v>All 7 sources are now graded, but 4 newly normalized series and EnterpriseArena each have one observation. Only Vending-Bench has a 3-point acceleration estimate. The Q3 drop is broader benchmark coverage, not frontier regression.</x:v>
+      </x:c>
+      <x:c r="J39" s="17"/>
+      <x:c r="K39" s="17"/>
+      <x:c r="L39" s="17"/>
+      <x:c r="M39" s="17"/>
+      <x:c r="N39" s="17"/>
+      <x:c r="O39" s="17"/>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="17" t="str">
@@ -1834,7 +1945,7 @@
       </x:c>
       <x:c r="B40" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AO$6:$AO$28),"")</x:f>
-        <x:v>0.34049947926846125</x:v>
+        <x:v>0.41596871174719136</x:v>
       </x:c>
       <x:c r="C40" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AO$6:$AO$28),"")</x:f>
@@ -1850,8 +1961,20 @@
       </x:c>
       <x:c r="F40" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B40:E40),"")</x:f>
-        <x:v>0.6200323528644938</x:v>
-      </x:c>
+        <x:v>0.6388996609841763</x:v>
+      </x:c>
+      <x:c r="H40" s="17" t="str">
+        <x:v>Ungraded</x:v>
+      </x:c>
+      <x:c r="I40" s="17" t="str">
+        <x:v>Blank score history means the benchmark lacks a defensible normalized observation.</x:v>
+      </x:c>
+      <x:c r="J40" s="17"/>
+      <x:c r="K40" s="17"/>
+      <x:c r="L40" s="17"/>
+      <x:c r="M40" s="17"/>
+      <x:c r="N40" s="17"/>
+      <x:c r="O40" s="17"/>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="17" t="str">
@@ -1859,7 +1982,7 @@
       </x:c>
       <x:c r="B41" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,B$21,'Report Card'!$AQ$6:$AQ$28),"")</x:f>
-        <x:v>0.34188613611131996</x:v>
+        <x:v>0.41656299325127366</x:v>
       </x:c>
       <x:c r="C41" s="19" t="n">
         <x:f>IFERROR(AVERAGEIF('Report Card'!$A$6:$A$28,C$21,'Report Card'!$AQ$6:$AQ$28),"")</x:f>
@@ -1875,8 +1998,20 @@
       </x:c>
       <x:c r="F41" s="19" t="n">
         <x:f>IFERROR(AVERAGE(B41:E41),"")</x:f>
-        <x:v>0.6233766173378316</x:v>
-      </x:c>
+        <x:v>0.6420458316228199</x:v>
+      </x:c>
+      <x:c r="H41" s="17" t="str">
+        <x:v>Caution</x:v>
+      </x:c>
+      <x:c r="I41" s="17" t="str">
+        <x:v>Sparse series project flat or constant velocity. This is a scenario, not a calibrated probability.</x:v>
+      </x:c>
+      <x:c r="J41" s="17"/>
+      <x:c r="K41" s="17"/>
+      <x:c r="L41" s="17"/>
+      <x:c r="M41" s="17"/>
+      <x:c r="N41" s="17"/>
+      <x:c r="O41" s="17"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1892,7 +2027,7 @@
     <x:mergeCell ref="G6:I9"/>
     <x:mergeCell ref="J6:L9"/>
     <x:mergeCell ref="M6:O9"/>
-    <x:mergeCell ref="A11:F11"/>
+    <x:mergeCell ref="A11:I11"/>
     <x:mergeCell ref="A20:F20"/>
     <x:mergeCell ref="H31:O31"/>
     <x:mergeCell ref="I32:O32"/>
@@ -1901,9 +2036,13 @@
     <x:mergeCell ref="I35:O35"/>
     <x:mergeCell ref="I36:O36"/>
     <x:mergeCell ref="I37:O37"/>
+    <x:mergeCell ref="I38:O38"/>
+    <x:mergeCell ref="I39:O39"/>
+    <x:mergeCell ref="I40:O40"/>
+    <x:mergeCell ref="I41:O41"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49c4d3ba866a47a8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5449359c135425f"/>
 </x:worksheet>
 </file>
 
@@ -2276,157 +2415,157 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="L3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="M3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="N3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="O3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="P3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="Q3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="R3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="S3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="T3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="U3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="V3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="W3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="X3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="Y3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="Z3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AA3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AB3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AC3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AD3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AE3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AF3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AG3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AH3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AI3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AJ3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AK3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AL3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AM3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AN3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AO3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AP3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AQ3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AR3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AS3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AT3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AU3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AV3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AW3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AX3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
       <x:c r="AY3" s="6" t="str">
-        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Rate is quarter-over-quarter score change. As of 2026-08-26.</x:v>
+        <x:v>Blue = observed release-quarter frontier; gray = carried frontier; gold = projected. Δ score is quarter-over-quarter percentage-point change; acceleration is failure-gap acceleration per quarter². As of 2026-08-26.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="32" hidden="0" customHeight="1">
@@ -2593,121 +2732,121 @@
         <x:v>Score</x:v>
       </x:c>
       <x:c r="F5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="G5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="H5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="J5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="K5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="L5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="M5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="N5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="O5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="P5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="Q5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="R5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="S5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="T5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="U5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="V5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="W5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="X5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="Y5" s="13" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="Z5" s="13" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AA5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AB5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AC5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AD5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AE5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AF5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AG5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AH5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AI5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AJ5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AK5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AL5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AM5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AN5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AO5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AP5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AQ5" s="27" t="str">
         <x:v>Score</x:v>
       </x:c>
       <x:c r="AR5" s="27" t="str">
-        <x:v>Rate</x:v>
+        <x:v>Δ score</x:v>
       </x:c>
       <x:c r="AS5" s="13" t="str">
         <x:v>Current Score</x:v>
@@ -2722,10 +2861,10 @@
         <x:v>Overall GPA</x:v>
       </x:c>
       <x:c r="AW5" s="13" t="str">
-        <x:v>Gap velocity / qtr</x:v>
+        <x:v>Gap velocity (halvings/qtr)</x:v>
       </x:c>
       <x:c r="AX5" s="13" t="str">
-        <x:v>Gap acceleration / qtr²</x:v>
+        <x:v>Gap acceleration (halvings/qtr²)</x:v>
       </x:c>
       <x:c r="AY5" s="13" t="str">
         <x:v>Projection basis</x:v>
@@ -3110,7 +3249,7 @@
         <x:v>YC-Bench</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>One-year startup final funds</x:v>
+        <x:v>Frontier mean final funds / $1M published substantial-profit threshold</x:v>
       </x:c>
       <x:c r="E8" s="43" t="str">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,"&lt;="&amp;1)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,"&lt;="&amp;1)))</x:f>
@@ -3166,81 +3305,104 @@
       <x:c r="V8" s="43" t="str">
         <x:f>IF(OR(U8="",S8=""),"",U8-S8)</x:f>
       </x:c>
-      <x:c r="W8" s="43" t="str">
+      <x:c r="W8" s="44" t="n">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,"&lt;="&amp;10)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,"&lt;="&amp;10)))</x:f>
-      </x:c>
-      <x:c r="X8" s="43" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="X8" s="44" t="str">
         <x:f>IF(OR(W8="",U8=""),"",W8-U8)</x:f>
       </x:c>
-      <x:c r="Y8" s="43" t="str">
+      <x:c r="Y8" s="43" t="n">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,"&lt;="&amp;11)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B8,'Observations'!$F$6:$F$500,"&lt;="&amp;11)))</x:f>
-      </x:c>
-      <x:c r="Z8" s="43" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Z8" s="43" t="n">
         <x:f>IF(OR(Y8="",W8=""),"",Y8-W8)</x:f>
-      </x:c>
-      <x:c r="AA8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AA8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(12-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(12-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AB8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AB8" s="45" t="n">
         <x:f>IF(OR(AA8="",Y8=""),"",AA8-Y8)</x:f>
-      </x:c>
-      <x:c r="AC8" s="45" t="str">
+        <x:v>-9.313225746154785e-10</x:v>
+      </x:c>
+      <x:c r="AC8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(13-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(13-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AD8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AD8" s="45" t="n">
         <x:f>IF(OR(AC8="",AA8=""),"",AC8-AA8)</x:f>
-      </x:c>
-      <x:c r="AE8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(14-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(14-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AF8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AF8" s="45" t="n">
         <x:f>IF(OR(AE8="",AC8=""),"",AE8-AC8)</x:f>
-      </x:c>
-      <x:c r="AG8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(15-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(15-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AH8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AH8" s="45" t="n">
         <x:f>IF(OR(AG8="",AE8=""),"",AG8-AE8)</x:f>
-      </x:c>
-      <x:c r="AI8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AI8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(16-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(16-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AJ8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AJ8" s="45" t="n">
         <x:f>IF(OR(AI8="",AG8=""),"",AI8-AG8)</x:f>
-      </x:c>
-      <x:c r="AK8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AK8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(17-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(17-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AL8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AL8" s="45" t="n">
         <x:f>IF(OR(AK8="",AI8=""),"",AK8-AI8)</x:f>
-      </x:c>
-      <x:c r="AM8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AM8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(18-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(18-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AN8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AN8" s="45" t="n">
         <x:f>IF(OR(AM8="",AK8=""),"",AM8-AK8)</x:f>
-      </x:c>
-      <x:c r="AO8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AO8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(19-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(19-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AP8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AP8" s="45" t="n">
         <x:f>IF(OR(AO8="",AM8=""),"",AO8-AM8)</x:f>
-      </x:c>
-      <x:c r="AQ8" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AQ8" s="45" t="n">
         <x:f>IF('Model'!$D8=0,"",1-POWER(2,-MAX('Model'!$M8,'Model'!$M8+'Model'!$N8*(20-'Methodology'!$B$8)+0.5*'Model'!$P8*POWER(20-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AR8" s="45" t="str">
+        <x:v>0.9999999990686774</x:v>
+      </x:c>
+      <x:c r="AR8" s="45" t="n">
         <x:f>IF(OR(AQ8="",AO8=""),"",AQ8-AO8)</x:f>
-      </x:c>
-      <x:c r="AS8" s="24" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS8" s="24" t="n">
         <x:f>IF('Model'!$D8=0,"",Y8)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AT8" s="17" t="str">
         <x:f>'Model'!S8</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="AU8" s="26" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="AU8" s="26" t="n">
         <x:f>IF('Model'!$D8=0,"",'Model'!T8)</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AV8" s="26" t="n">
         <x:f>AVERAGE(AVERAGEIF($A$6:$A$28,"Direct economic stewardship",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Operational execution",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Personal stewardship transfer",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Economic value &amp; governance",$AU$6:$AU$28))</x:f>
@@ -3256,7 +3418,7 @@
       </x:c>
       <x:c r="AY8" s="17" t="str">
         <x:f>'Model'!Q8</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
+        <x:v>Flat — one observation</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" hidden="0" customHeight="1">
@@ -3270,7 +3432,7 @@
         <x:v>Business Arena</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>30-day seller final worth</x:v>
+        <x:v>Best-model mean final worth / $436,195 expert-strategy final worth</x:v>
       </x:c>
       <x:c r="E9" s="43" t="str">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B9,'Observations'!$F$6:$F$500,"&lt;="&amp;1)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B9,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B9,'Observations'!$F$6:$F$500,"&lt;="&amp;1)))</x:f>
@@ -3332,75 +3494,96 @@
       <x:c r="X9" s="43" t="str">
         <x:f>IF(OR(W9="",U9=""),"",W9-U9)</x:f>
       </x:c>
-      <x:c r="Y9" s="43" t="str">
+      <x:c r="Y9" s="44" t="n">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B9,'Observations'!$F$6:$F$500,"&lt;="&amp;11)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B9,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B9,'Observations'!$F$6:$F$500,"&lt;="&amp;11)))</x:f>
-      </x:c>
-      <x:c r="Z9" s="43" t="str">
+        <x:v>0.4321186625247882</x:v>
+      </x:c>
+      <x:c r="Z9" s="44" t="str">
         <x:f>IF(OR(Y9="",W9=""),"",Y9-W9)</x:f>
       </x:c>
-      <x:c r="AA9" s="45" t="str">
+      <x:c r="AA9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(12-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(12-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AB9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AB9" s="45" t="n">
         <x:f>IF(OR(AA9="",Y9=""),"",AA9-Y9)</x:f>
-      </x:c>
-      <x:c r="AC9" s="45" t="str">
+        <x:v>-5.551115123125783e-17</x:v>
+      </x:c>
+      <x:c r="AC9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(13-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(13-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AD9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AD9" s="45" t="n">
         <x:f>IF(OR(AC9="",AA9=""),"",AC9-AA9)</x:f>
-      </x:c>
-      <x:c r="AE9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(14-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(14-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AF9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AF9" s="45" t="n">
         <x:f>IF(OR(AE9="",AC9=""),"",AE9-AC9)</x:f>
-      </x:c>
-      <x:c r="AG9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(15-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(15-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AH9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AH9" s="45" t="n">
         <x:f>IF(OR(AG9="",AE9=""),"",AG9-AE9)</x:f>
-      </x:c>
-      <x:c r="AI9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AI9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(16-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(16-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AJ9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AJ9" s="45" t="n">
         <x:f>IF(OR(AI9="",AG9=""),"",AI9-AG9)</x:f>
-      </x:c>
-      <x:c r="AK9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AK9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(17-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(17-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AL9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AL9" s="45" t="n">
         <x:f>IF(OR(AK9="",AI9=""),"",AK9-AI9)</x:f>
-      </x:c>
-      <x:c r="AM9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AM9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(18-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(18-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AN9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AN9" s="45" t="n">
         <x:f>IF(OR(AM9="",AK9=""),"",AM9-AK9)</x:f>
-      </x:c>
-      <x:c r="AO9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AO9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(19-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(19-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AP9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AP9" s="45" t="n">
         <x:f>IF(OR(AO9="",AM9=""),"",AO9-AM9)</x:f>
-      </x:c>
-      <x:c r="AQ9" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AQ9" s="45" t="n">
         <x:f>IF('Model'!$D9=0,"",1-POWER(2,-MAX('Model'!$M9,'Model'!$M9+'Model'!$N9*(20-'Methodology'!$B$8)+0.5*'Model'!$P9*POWER(20-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AR9" s="45" t="str">
+        <x:v>0.43211866252478814</x:v>
+      </x:c>
+      <x:c r="AR9" s="45" t="n">
         <x:f>IF(OR(AQ9="",AO9=""),"",AQ9-AO9)</x:f>
-      </x:c>
-      <x:c r="AS9" s="24" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS9" s="24" t="n">
         <x:f>IF('Model'!$D9=0,"",Y9)</x:f>
+        <x:v>0.4321186625247882</x:v>
       </x:c>
       <x:c r="AT9" s="17" t="str">
         <x:f>'Model'!S9</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="AU9" s="26" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="AU9" s="26" t="n">
         <x:f>IF('Model'!$D9=0,"",'Model'!T9)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV9" s="26" t="n">
         <x:f>AVERAGE(AVERAGEIF($A$6:$A$28,"Direct economic stewardship",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Operational execution",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Personal stewardship transfer",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Economic value &amp; governance",$AU$6:$AU$28))</x:f>
@@ -3416,7 +3599,7 @@
       </x:c>
       <x:c r="AY9" s="17" t="str">
         <x:f>'Model'!Q9</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
+        <x:v>Flat — one observation</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" hidden="0" customHeight="1">
@@ -3615,7 +3798,7 @@
         <x:v>RetailBench</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str">
-        <x:v>Long-horizon retail operations score</x:v>
+        <x:v>Best LLM final net worth / $131,510.42 oracle final net worth</x:v>
       </x:c>
       <x:c r="E11" s="43" t="str">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B11,'Observations'!$F$6:$F$500,"&lt;="&amp;1)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B11,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B11,'Observations'!$F$6:$F$500,"&lt;="&amp;1)))</x:f>
@@ -3677,75 +3860,96 @@
       <x:c r="X11" s="43" t="str">
         <x:f>IF(OR(W11="",U11=""),"",W11-U11)</x:f>
       </x:c>
-      <x:c r="Y11" s="43" t="str">
+      <x:c r="Y11" s="44" t="n">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B11,'Observations'!$F$6:$F$500,"&lt;="&amp;11)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B11,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B11,'Observations'!$F$6:$F$500,"&lt;="&amp;11)))</x:f>
-      </x:c>
-      <x:c r="Z11" s="43" t="str">
+        <x:v>0.18516388283148968</x:v>
+      </x:c>
+      <x:c r="Z11" s="44" t="str">
         <x:f>IF(OR(Y11="",W11=""),"",Y11-W11)</x:f>
       </x:c>
-      <x:c r="AA11" s="45" t="str">
+      <x:c r="AA11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(12-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(12-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AB11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AB11" s="45" t="n">
         <x:f>IF(OR(AA11="",Y11=""),"",AA11-Y11)</x:f>
-      </x:c>
-      <x:c r="AC11" s="45" t="str">
+        <x:v>-2.7755575615628914e-17</x:v>
+      </x:c>
+      <x:c r="AC11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(13-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(13-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AD11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AD11" s="45" t="n">
         <x:f>IF(OR(AC11="",AA11=""),"",AC11-AA11)</x:f>
-      </x:c>
-      <x:c r="AE11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(14-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(14-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AF11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AF11" s="45" t="n">
         <x:f>IF(OR(AE11="",AC11=""),"",AE11-AC11)</x:f>
-      </x:c>
-      <x:c r="AG11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(15-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(15-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AH11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AH11" s="45" t="n">
         <x:f>IF(OR(AG11="",AE11=""),"",AG11-AE11)</x:f>
-      </x:c>
-      <x:c r="AI11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AI11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(16-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(16-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AJ11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AJ11" s="45" t="n">
         <x:f>IF(OR(AI11="",AG11=""),"",AI11-AG11)</x:f>
-      </x:c>
-      <x:c r="AK11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AK11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(17-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(17-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AL11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AL11" s="45" t="n">
         <x:f>IF(OR(AK11="",AI11=""),"",AK11-AI11)</x:f>
-      </x:c>
-      <x:c r="AM11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AM11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(18-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(18-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AN11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AN11" s="45" t="n">
         <x:f>IF(OR(AM11="",AK11=""),"",AM11-AK11)</x:f>
-      </x:c>
-      <x:c r="AO11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AO11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(19-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(19-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AP11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AP11" s="45" t="n">
         <x:f>IF(OR(AO11="",AM11=""),"",AO11-AM11)</x:f>
-      </x:c>
-      <x:c r="AQ11" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AQ11" s="45" t="n">
         <x:f>IF('Model'!$D11=0,"",1-POWER(2,-MAX('Model'!$M11,'Model'!$M11+'Model'!$N11*(20-'Methodology'!$B$8)+0.5*'Model'!$P11*POWER(20-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AR11" s="45" t="str">
+        <x:v>0.18516388283148966</x:v>
+      </x:c>
+      <x:c r="AR11" s="45" t="n">
         <x:f>IF(OR(AQ11="",AO11=""),"",AQ11-AO11)</x:f>
-      </x:c>
-      <x:c r="AS11" s="24" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS11" s="24" t="n">
         <x:f>IF('Model'!$D11=0,"",Y11)</x:f>
+        <x:v>0.18516388283148968</x:v>
       </x:c>
       <x:c r="AT11" s="17" t="str">
         <x:f>'Model'!S11</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="AU11" s="26" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="AU11" s="26" t="n">
         <x:f>IF('Model'!$D11=0,"",'Model'!T11)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV11" s="26" t="n">
         <x:f>AVERAGE(AVERAGEIF($A$6:$A$28,"Direct economic stewardship",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Operational execution",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Personal stewardship transfer",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Economic value &amp; governance",$AU$6:$AU$28))</x:f>
@@ -3761,7 +3965,7 @@
       </x:c>
       <x:c r="AY11" s="17" t="str">
         <x:f>'Model'!Q11</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
+        <x:v>Flat — one observation</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" hidden="0" customHeight="1">
@@ -3775,7 +3979,7 @@
         <x:v>MerchantBench</x:v>
       </x:c>
       <x:c r="D12" s="17" t="str">
-        <x:v>365-day ecommerce operating score</x:v>
+        <x:v>Best LLM mean final net assets / human-participant mean</x:v>
       </x:c>
       <x:c r="E12" s="43" t="str">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B12,'Observations'!$F$6:$F$500,"&lt;="&amp;1)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B12,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B12,'Observations'!$F$6:$F$500,"&lt;="&amp;1)))</x:f>
@@ -3837,75 +4041,96 @@
       <x:c r="X12" s="43" t="str">
         <x:f>IF(OR(W12="",U12=""),"",W12-U12)</x:f>
       </x:c>
-      <x:c r="Y12" s="43" t="str">
+      <x:c r="Y12" s="44" t="n">
         <x:f>IF(COUNTIFS('Observations'!$A$6:$A$500,$B12,'Observations'!$F$6:$F$500,"&lt;="&amp;11)=0,"",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,$B12,'Observations'!$F$6:$F$500,MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,$B12,'Observations'!$F$6:$F$500,"&lt;="&amp;11)))</x:f>
-      </x:c>
-      <x:c r="Z12" s="43" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="Z12" s="44" t="str">
         <x:f>IF(OR(Y12="",W12=""),"",Y12-W12)</x:f>
       </x:c>
-      <x:c r="AA12" s="45" t="str">
+      <x:c r="AA12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(12-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(12-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AB12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AB12" s="45" t="n">
         <x:f>IF(OR(AA12="",Y12=""),"",AA12-Y12)</x:f>
-      </x:c>
-      <x:c r="AC12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AC12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(13-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(13-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AD12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AD12" s="45" t="n">
         <x:f>IF(OR(AC12="",AA12=""),"",AC12-AA12)</x:f>
-      </x:c>
-      <x:c r="AE12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AE12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(14-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(14-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AF12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AF12" s="45" t="n">
         <x:f>IF(OR(AE12="",AC12=""),"",AE12-AC12)</x:f>
-      </x:c>
-      <x:c r="AG12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AG12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(15-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(15-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AH12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AH12" s="45" t="n">
         <x:f>IF(OR(AG12="",AE12=""),"",AG12-AE12)</x:f>
-      </x:c>
-      <x:c r="AI12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AI12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(16-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(16-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AJ12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AJ12" s="45" t="n">
         <x:f>IF(OR(AI12="",AG12=""),"",AI12-AG12)</x:f>
-      </x:c>
-      <x:c r="AK12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AK12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(17-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(17-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AL12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AL12" s="45" t="n">
         <x:f>IF(OR(AK12="",AI12=""),"",AK12-AI12)</x:f>
-      </x:c>
-      <x:c r="AM12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AM12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(18-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(18-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AN12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AN12" s="45" t="n">
         <x:f>IF(OR(AM12="",AK12=""),"",AM12-AK12)</x:f>
-      </x:c>
-      <x:c r="AO12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AO12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(19-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(19-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AP12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AP12" s="45" t="n">
         <x:f>IF(OR(AO12="",AM12=""),"",AO12-AM12)</x:f>
-      </x:c>
-      <x:c r="AQ12" s="45" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AQ12" s="45" t="n">
         <x:f>IF('Model'!$D12=0,"",1-POWER(2,-MAX('Model'!$M12,'Model'!$M12+'Model'!$N12*(20-'Methodology'!$B$8)+0.5*'Model'!$P12*POWER(20-'Methodology'!$B$8,2))))</x:f>
-      </x:c>
-      <x:c r="AR12" s="45" t="str">
+        <x:v>0.273</x:v>
+      </x:c>
+      <x:c r="AR12" s="45" t="n">
         <x:f>IF(OR(AQ12="",AO12=""),"",AQ12-AO12)</x:f>
-      </x:c>
-      <x:c r="AS12" s="24" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AS12" s="24" t="n">
         <x:f>IF('Model'!$D12=0,"",Y12)</x:f>
+        <x:v>0.273</x:v>
       </x:c>
       <x:c r="AT12" s="17" t="str">
         <x:f>'Model'!S12</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="AU12" s="26" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="AU12" s="26" t="n">
         <x:f>IF('Model'!$D12=0,"",'Model'!T12)</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV12" s="26" t="n">
         <x:f>AVERAGE(AVERAGEIF($A$6:$A$28,"Direct economic stewardship",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Operational execution",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Personal stewardship transfer",$AU$6:$AU$28),AVERAGEIF($A$6:$A$28,"Economic value &amp; governance",$AU$6:$AU$28))</x:f>
@@ -3921,7 +4146,7 @@
       </x:c>
       <x:c r="AY12" s="17" t="str">
         <x:f>'Model'!Q12</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
+        <x:v>Flat — one observation</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" hidden="0" customHeight="1">
@@ -6985,37 +7210,37 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str">
-        <x:v>Append-only evidence ledger. Score must be a defensible 0–100% completion/saturation measure; do not enter Elo or raw dollars without a published target.</x:v>
+        <x:v>Append-only evidence ledger. Raw dollars and Elo enter the report only after conversion against a fixed, sourced target or reference anchor.</x:v>
       </x:c>
     </x:row>
     <x:row r="4"/>
@@ -7229,249 +7454,249 @@
         <x:v>Three runs/model; best-run statistic is noisy.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="17" t="str">
-        <x:v>DES-05</x:v>
+        <x:v>DES-03</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>EnterpriseArena</x:v>
+        <x:v>YC-Bench</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
         <x:v>Direct economic stewardship</x:v>
       </x:c>
       <x:c r="D11" s="18" t="n">
-        <x:v>46101</x:v>
+        <x:v>46113</x:v>
       </x:c>
       <x:c r="E11" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2026-Q2</x:v>
       </x:c>
       <x:c r="F11" s="17" t="n">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G11" s="24" t="n">
-        <x:v>0.8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="17" t="str">
-        <x:v>Qwen 3.5 9B</x:v>
+        <x:v>Claude Opus 4.6</x:v>
       </x:c>
       <x:c r="I11" s="17" t="str">
-        <x:v>Best-model full-horizon survival</x:v>
+        <x:v>Mean final funds / $1M published substantial-profit threshold</x:v>
       </x:c>
       <x:c r="J11" s="17" t="str">
-        <x:v>https://arxiv.org/abs/2603.23638</x:v>
+        <x:v>https://arxiv.org/abs/2604.01212</x:v>
       </x:c>
       <x:c r="K11" s="17" t="str">
-        <x:v>Single launch-era frontier; flat forecast until another comparable point.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>Provisional target-normalized score. Saturated at launch; no human or oracle ceiling is published.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A12" s="17" t="str">
-        <x:v>OPS-01</x:v>
+        <x:v>DES-04</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>AutomationBench</x:v>
+        <x:v>Business Arena</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>Operational execution</x:v>
+        <x:v>Direct economic stewardship</x:v>
       </x:c>
       <x:c r="D12" s="18" t="n">
-        <x:v>46182</x:v>
+        <x:v>46245</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:v>2026-Q2</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="F12" s="17" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G12" s="24" t="n">
-        <x:v>0.4617</x:v>
+        <x:v>0.4321186625247882</x:v>
       </x:c>
       <x:c r="H12" s="17" t="str">
-        <x:v>Claude Fable 5</x:v>
+        <x:v>Gemini 3.1 Pro</x:v>
       </x:c>
       <x:c r="I12" s="17" t="str">
-        <x:v>Public 600-task pass rate, max reasoning</x:v>
+        <x:v>Best-model mean final worth / expert-strategy final worth</x:v>
       </x:c>
       <x:c r="J12" s="17" t="str">
-        <x:v>https://github.com/zapier/AutomationBench</x:v>
+        <x:v>https://arxiv.org/abs/2608.08621</x:v>
       </x:c>
       <x:c r="K12" s="17" t="str">
-        <x:v>Score rerun under the July 2026 stricter classifier.</x:v>
+        <x:v>Ten matched runs per model; reference strategy uses only agent-visible information.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="17" t="str">
-        <x:v>OPS-01</x:v>
+        <x:v>DES-05</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>AutomationBench</x:v>
+        <x:v>EnterpriseArena</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
-        <x:v>Operational execution</x:v>
+        <x:v>Direct economic stewardship</x:v>
       </x:c>
       <x:c r="D13" s="18" t="n">
-        <x:v>46227</x:v>
+        <x:v>46101</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="F13" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G13" s="24" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="H13" s="17" t="str">
+        <x:v>Qwen 3.5 9B</x:v>
+      </x:c>
+      <x:c r="I13" s="17" t="str">
+        <x:v>Best-model full-horizon survival</x:v>
+      </x:c>
+      <x:c r="J13" s="17" t="str">
+        <x:v>https://arxiv.org/abs/2603.23638</x:v>
+      </x:c>
+      <x:c r="K13" s="17" t="str">
+        <x:v>Single launch-era frontier; flat forecast until another comparable point.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A14" s="17" t="str">
+        <x:v>DES-06</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>RetailBench</x:v>
+      </x:c>
+      <x:c r="C14" s="17" t="str">
+        <x:v>Direct economic stewardship</x:v>
+      </x:c>
+      <x:c r="D14" s="18" t="n">
+        <x:v>46211</x:v>
+      </x:c>
+      <x:c r="E14" s="17" t="str">
         <x:v>2026-Q3</x:v>
       </x:c>
-      <x:c r="F13" s="17" t="n">
+      <x:c r="F14" s="17" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G13" s="24" t="n">
-        <x:v>0.503</x:v>
-      </x:c>
-      <x:c r="H13" s="17" t="str">
-        <x:v>Claude Opus 5</x:v>
-      </x:c>
-      <x:c r="I13" s="17" t="str">
-        <x:v>Public 600-task pass rate, max reasoning</x:v>
-      </x:c>
-      <x:c r="J13" s="17" t="str">
-        <x:v>https://github.com/zapier/AutomationBench</x:v>
-      </x:c>
-      <x:c r="K13" s="17" t="str">
-        <x:v>Current public frontier.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="17" t="str">
-        <x:v>OPS-02</x:v>
-      </x:c>
-      <x:c r="B14" s="17" t="str">
-        <x:v>EnterpriseOps-Gym</x:v>
-      </x:c>
-      <x:c r="C14" s="17" t="str">
-        <x:v>Operational execution</x:v>
-      </x:c>
-      <x:c r="D14" s="18" t="n">
-        <x:v>45825</x:v>
-      </x:c>
-      <x:c r="E14" s="17" t="str">
-        <x:v>2025-Q2</x:v>
-      </x:c>
-      <x:c r="F14" s="17" t="n">
-        <x:v>6</x:v>
-      </x:c>
       <x:c r="G14" s="24" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.18516388283148968</x:v>
       </x:c>
       <x:c r="H14" s="17" t="str">
-        <x:v>Gemini 2.5 Pro</x:v>
+        <x:v>GPT-5.5 + ReAct</x:v>
       </x:c>
       <x:c r="I14" s="17" t="str">
-        <x:v>Strict task success</x:v>
+        <x:v>Best LLM final net worth / oracle final net worth</x:v>
       </x:c>
       <x:c r="J14" s="17" t="str">
-        <x:v>https://enterpriseops-gym.github.io/</x:v>
+        <x:v>https://arxiv.org/abs/2603.16453</x:v>
       </x:c>
       <x:c r="K14" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+        <x:v>Selected-run protocol; oracle has privileged simulator access and is a ceiling-like reference.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A15" s="17" t="str">
-        <x:v>OPS-02</x:v>
+        <x:v>DES-07</x:v>
       </x:c>
       <x:c r="B15" s="17" t="str">
-        <x:v>EnterpriseOps-Gym</x:v>
+        <x:v>MerchantBench</x:v>
       </x:c>
       <x:c r="C15" s="17" t="str">
-        <x:v>Operational execution</x:v>
+        <x:v>Direct economic stewardship</x:v>
       </x:c>
       <x:c r="D15" s="18" t="n">
-        <x:v>45929</x:v>
+        <x:v>46238</x:v>
       </x:c>
       <x:c r="E15" s="17" t="str">
-        <x:v>2025-Q3</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="F15" s="17" t="n">
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G15" s="24" t="n">
-        <x:v>0.341</x:v>
+        <x:v>0.273</x:v>
       </x:c>
       <x:c r="H15" s="17" t="str">
-        <x:v>Claude Sonnet 4.5</x:v>
+        <x:v>Qwen3.7-Max + Hermes</x:v>
       </x:c>
       <x:c r="I15" s="17" t="str">
-        <x:v>Strict task success</x:v>
+        <x:v>Best LLM mean final net assets / human mean</x:v>
       </x:c>
       <x:c r="J15" s="17" t="str">
-        <x:v>https://enterpriseops-gym.github.io/</x:v>
+        <x:v>https://arxiv.org/abs/2607.28956</x:v>
       </x:c>
       <x:c r="K15" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Authors' reported ratio; three LLM runs per configuration and three non-expert human participants.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
-        <x:v>OPS-02</x:v>
+        <x:v>OPS-01</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
-        <x:v>EnterpriseOps-Gym</x:v>
+        <x:v>AutomationBench</x:v>
       </x:c>
       <x:c r="C16" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D16" s="18" t="n">
-        <x:v>45985</x:v>
+        <x:v>46182</x:v>
       </x:c>
       <x:c r="E16" s="17" t="str">
-        <x:v>2025-Q4</x:v>
+        <x:v>2026-Q2</x:v>
       </x:c>
       <x:c r="F16" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G16" s="24" t="n">
-        <x:v>0.394</x:v>
+        <x:v>0.4617</x:v>
       </x:c>
       <x:c r="H16" s="17" t="str">
-        <x:v>Claude Opus 4.5</x:v>
+        <x:v>Claude Fable 5</x:v>
       </x:c>
       <x:c r="I16" s="17" t="str">
-        <x:v>Strict task success</x:v>
+        <x:v>Public 600-task pass rate, max reasoning</x:v>
       </x:c>
       <x:c r="J16" s="17" t="str">
-        <x:v>https://enterpriseops-gym.github.io/</x:v>
+        <x:v>https://github.com/zapier/AutomationBench</x:v>
       </x:c>
       <x:c r="K16" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Score rerun under the July 2026 stricter classifier.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="17" t="str">
-        <x:v>OPS-02</x:v>
+        <x:v>OPS-01</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
-        <x:v>EnterpriseOps-Gym</x:v>
+        <x:v>AutomationBench</x:v>
       </x:c>
       <x:c r="C17" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D17" s="18" t="n">
-        <x:v>46058</x:v>
+        <x:v>46227</x:v>
       </x:c>
       <x:c r="E17" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="F17" s="17" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G17" s="24" t="n">
-        <x:v>0.459</x:v>
+        <x:v>0.503</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
-        <x:v>Claude Opus 4.6</x:v>
+        <x:v>Claude Opus 5</x:v>
       </x:c>
       <x:c r="I17" s="17" t="str">
-        <x:v>Strict task success</x:v>
+        <x:v>Public 600-task pass rate, max reasoning</x:v>
       </x:c>
       <x:c r="J17" s="17" t="str">
-        <x:v>https://enterpriseops-gym.github.io/</x:v>
+        <x:v>https://github.com/zapier/AutomationBench</x:v>
       </x:c>
       <x:c r="K17" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Current public frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -7485,19 +7710,19 @@
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D18" s="18" t="n">
-        <x:v>46204</x:v>
+        <x:v>45825</x:v>
       </x:c>
       <x:c r="E18" s="17" t="str">
-        <x:v>2026-Q3</x:v>
+        <x:v>2025-Q2</x:v>
       </x:c>
       <x:c r="F18" s="17" t="n">
-        <x:v>11</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G18" s="24" t="n">
-        <x:v>0.511</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="H18" s="17" t="str">
-        <x:v>Claude Fable 5 + fallback</x:v>
+        <x:v>Gemini 2.5 Pro</x:v>
       </x:c>
       <x:c r="I18" s="17" t="str">
         <x:v>Strict task success</x:v>
@@ -7506,427 +7731,427 @@
         <x:v>https://enterpriseops-gym.github.io/</x:v>
       </x:c>
       <x:c r="K18" s="17" t="str">
-        <x:v>Harness includes fallback; pin this configuration for future comparison.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="17" t="str">
-        <x:v>OPS-03</x:v>
+        <x:v>OPS-02</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>Commerce Agent Bench</x:v>
+        <x:v>EnterpriseOps-Gym</x:v>
       </x:c>
       <x:c r="C19" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D19" s="18" t="n">
-        <x:v>46008</x:v>
+        <x:v>45929</x:v>
       </x:c>
       <x:c r="E19" s="17" t="str">
-        <x:v>2025-Q4</x:v>
+        <x:v>2025-Q3</x:v>
       </x:c>
       <x:c r="F19" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G19" s="24" t="n">
-        <x:v>0.29</x:v>
+        <x:v>0.341</x:v>
       </x:c>
       <x:c r="H19" s="17" t="str">
-        <x:v>Gemini 3 Flash + Pi</x:v>
+        <x:v>Claude Sonnet 4.5</x:v>
       </x:c>
       <x:c r="I19" s="17" t="str">
-        <x:v>Pi-harness full-suite pass rate</x:v>
+        <x:v>Strict task success</x:v>
       </x:c>
       <x:c r="J19" s="17" t="str">
-        <x:v>https://github.com/Accio-org/CommerceAgentBench</x:v>
+        <x:v>https://enterpriseops-gym.github.io/</x:v>
       </x:c>
       <x:c r="K19" s="17" t="str">
-        <x:v>107-task benchmark snapshot.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="17" t="str">
-        <x:v>OPS-03</x:v>
+        <x:v>OPS-02</x:v>
       </x:c>
       <x:c r="B20" s="17" t="str">
-        <x:v>Commerce Agent Bench</x:v>
+        <x:v>EnterpriseOps-Gym</x:v>
       </x:c>
       <x:c r="C20" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D20" s="18" t="n">
-        <x:v>46143</x:v>
+        <x:v>45985</x:v>
       </x:c>
       <x:c r="E20" s="17" t="str">
-        <x:v>2026-Q2</x:v>
+        <x:v>2025-Q4</x:v>
       </x:c>
       <x:c r="F20" s="17" t="n">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G20" s="24" t="n">
-        <x:v>0.523</x:v>
+        <x:v>0.394</x:v>
       </x:c>
       <x:c r="H20" s="17" t="str">
-        <x:v>Claude Opus 4.8 + Pi</x:v>
+        <x:v>Claude Opus 4.5</x:v>
       </x:c>
       <x:c r="I20" s="17" t="str">
-        <x:v>Pi-harness full-suite pass rate</x:v>
+        <x:v>Strict task success</x:v>
       </x:c>
       <x:c r="J20" s="17" t="str">
-        <x:v>https://github.com/Accio-org/CommerceAgentBench</x:v>
+        <x:v>https://enterpriseops-gym.github.io/</x:v>
       </x:c>
       <x:c r="K20" s="17" t="str">
-        <x:v>Quarter frontier; fixed Pi harness.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="17" t="str">
-        <x:v>OPS-03</x:v>
+        <x:v>OPS-02</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>Commerce Agent Bench</x:v>
+        <x:v>EnterpriseOps-Gym</x:v>
       </x:c>
       <x:c r="C21" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D21" s="18" t="n">
-        <x:v>46227</x:v>
+        <x:v>46058</x:v>
       </x:c>
       <x:c r="E21" s="17" t="str">
-        <x:v>2026-Q3</x:v>
+        <x:v>2026-Q1</x:v>
       </x:c>
       <x:c r="F21" s="17" t="n">
-        <x:v>11</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G21" s="24" t="n">
-        <x:v>0.607</x:v>
+        <x:v>0.459</x:v>
       </x:c>
       <x:c r="H21" s="17" t="str">
-        <x:v>Claude Opus 5 + Pi</x:v>
+        <x:v>Claude Opus 4.6</x:v>
       </x:c>
       <x:c r="I21" s="17" t="str">
-        <x:v>Pi-harness full-suite pass rate</x:v>
+        <x:v>Strict task success</x:v>
       </x:c>
       <x:c r="J21" s="17" t="str">
-        <x:v>https://github.com/Accio-org/CommerceAgentBench</x:v>
+        <x:v>https://enterpriseops-gym.github.io/</x:v>
       </x:c>
       <x:c r="K21" s="17" t="str">
-        <x:v>65/107 tasks; fixed Pi harness.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="17" t="str">
-        <x:v>OPS-04</x:v>
+        <x:v>OPS-02</x:v>
       </x:c>
       <x:c r="B22" s="17" t="str">
-        <x:v>ClawMark</x:v>
+        <x:v>EnterpriseOps-Gym</x:v>
       </x:c>
       <x:c r="C22" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D22" s="18" t="n">
-        <x:v>46082</x:v>
+        <x:v>46204</x:v>
       </x:c>
       <x:c r="E22" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="F22" s="17" t="n">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G22" s="24" t="n">
-        <x:v>0.758</x:v>
+        <x:v>0.511</x:v>
       </x:c>
       <x:c r="H22" s="17" t="str">
-        <x:v>Claude Sonnet 4.6</x:v>
+        <x:v>Claude Fable 5 + fallback</x:v>
       </x:c>
       <x:c r="I22" s="17" t="str">
-        <x:v>Avg@3 weighted deterministic-checker score</x:v>
+        <x:v>Strict task success</x:v>
       </x:c>
       <x:c r="J22" s="17" t="str">
-        <x:v>https://github.com/evolvent-ai/ClawMark</x:v>
+        <x:v>https://enterpriseops-gym.github.io/</x:v>
       </x:c>
       <x:c r="K22" s="17" t="str">
-        <x:v>One pinned 100-task repo snapshot.</x:v>
+        <x:v>Harness includes fallback; pin this configuration for future comparison.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="17" t="str">
-        <x:v>OPS-05</x:v>
+        <x:v>OPS-03</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
-        <x:v>TheAgentCompany</x:v>
+        <x:v>Commerce Agent Bench</x:v>
       </x:c>
       <x:c r="C23" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D23" s="18" t="n">
-        <x:v>45645</x:v>
+        <x:v>46008</x:v>
       </x:c>
       <x:c r="E23" s="17" t="str">
-        <x:v>2024-Q4</x:v>
+        <x:v>2025-Q4</x:v>
       </x:c>
       <x:c r="F23" s="17" t="n">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G23" s="24" t="n">
-        <x:v>0.24</x:v>
+        <x:v>0.29</x:v>
       </x:c>
       <x:c r="H23" s="17" t="str">
-        <x:v>Launch-paper best system</x:v>
+        <x:v>Gemini 3 Flash + Pi</x:v>
       </x:c>
       <x:c r="I23" s="17" t="str">
-        <x:v>Fraction of tasks completed</x:v>
+        <x:v>Pi-harness full-suite pass rate</x:v>
       </x:c>
       <x:c r="J23" s="17" t="str">
-        <x:v>https://arxiv.org/abs/2412.14161</x:v>
+        <x:v>https://github.com/Accio-org/CommerceAgentBench</x:v>
       </x:c>
       <x:c r="K23" s="17" t="str">
-        <x:v>Primary-paper baseline.</x:v>
+        <x:v>107-task benchmark snapshot.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="17" t="str">
-        <x:v>OPS-05</x:v>
+        <x:v>OPS-03</x:v>
       </x:c>
       <x:c r="B24" s="17" t="str">
-        <x:v>TheAgentCompany</x:v>
+        <x:v>Commerce Agent Bench</x:v>
       </x:c>
       <x:c r="C24" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D24" s="18" t="n">
-        <x:v>45825</x:v>
+        <x:v>46143</x:v>
       </x:c>
       <x:c r="E24" s="17" t="str">
-        <x:v>2025-Q2</x:v>
+        <x:v>2026-Q2</x:v>
       </x:c>
       <x:c r="F24" s="17" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G24" s="24" t="n">
-        <x:v>0.303</x:v>
+        <x:v>0.523</x:v>
       </x:c>
       <x:c r="H24" s="17" t="str">
-        <x:v>Gemini 2.5 Pro</x:v>
+        <x:v>Claude Opus 4.8 + Pi</x:v>
       </x:c>
       <x:c r="I24" s="17" t="str">
-        <x:v>Fraction of tasks completed</x:v>
+        <x:v>Pi-harness full-suite pass rate</x:v>
       </x:c>
       <x:c r="J24" s="17" t="str">
-        <x:v>https://the-agent-company.com/</x:v>
+        <x:v>https://github.com/Accio-org/CommerceAgentBench</x:v>
       </x:c>
       <x:c r="K24" s="17" t="str">
-        <x:v>Later leaderboard configuration; comparability caveat.</x:v>
+        <x:v>Quarter frontier; fixed Pi harness.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="17" t="str">
-        <x:v>OPS-05</x:v>
+        <x:v>OPS-03</x:v>
       </x:c>
       <x:c r="B25" s="17" t="str">
-        <x:v>TheAgentCompany</x:v>
+        <x:v>Commerce Agent Bench</x:v>
       </x:c>
       <x:c r="C25" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D25" s="18" t="n">
-        <x:v>45901</x:v>
+        <x:v>46227</x:v>
       </x:c>
       <x:c r="E25" s="17" t="str">
-        <x:v>2025-Q3</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="F25" s="17" t="n">
-        <x:v>7</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G25" s="24" t="n">
-        <x:v>0.429</x:v>
+        <x:v>0.607</x:v>
       </x:c>
       <x:c r="H25" s="17" t="str">
-        <x:v>DeepSeek V3.2 + specialized harness</x:v>
+        <x:v>Claude Opus 5 + Pi</x:v>
       </x:c>
       <x:c r="I25" s="17" t="str">
-        <x:v>Fraction of tasks completed</x:v>
+        <x:v>Pi-harness full-suite pass rate</x:v>
       </x:c>
       <x:c r="J25" s="17" t="str">
-        <x:v>https://the-agent-company.com/</x:v>
+        <x:v>https://github.com/Accio-org/CommerceAgentBench</x:v>
       </x:c>
       <x:c r="K25" s="17" t="str">
-        <x:v>Community/specialized harness; system-level frontier.</x:v>
+        <x:v>65/107 tasks; fixed Pi harness.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="17" t="str">
-        <x:v>OPS-07</x:v>
+        <x:v>OPS-04</x:v>
       </x:c>
       <x:c r="B26" s="17" t="str">
-        <x:v>Finch / FinWorkBench</x:v>
+        <x:v>ClawMark</x:v>
       </x:c>
       <x:c r="C26" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D26" s="18" t="n">
-        <x:v>45974</x:v>
+        <x:v>46082</x:v>
       </x:c>
       <x:c r="E26" s="17" t="str">
-        <x:v>2025-Q4</x:v>
+        <x:v>2026-Q1</x:v>
       </x:c>
       <x:c r="F26" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G26" s="24" t="n">
-        <x:v>0.384</x:v>
+        <x:v>0.758</x:v>
       </x:c>
       <x:c r="H26" s="17" t="str">
-        <x:v>GPT-5.1 Pro</x:v>
+        <x:v>Claude Sonnet 4.6</x:v>
       </x:c>
       <x:c r="I26" s="17" t="str">
-        <x:v>Strict finance-work task pass rate</x:v>
+        <x:v>Avg@3 weighted deterministic-checker score</x:v>
       </x:c>
       <x:c r="J26" s="17" t="str">
-        <x:v>https://aclanthology.org/2026.findings-acl.523/</x:v>
+        <x:v>https://github.com/evolvent-ai/ClawMark</x:v>
       </x:c>
       <x:c r="K26" s="17" t="str">
-        <x:v>Model release-quarter assignment; publication followed in 2026.</x:v>
+        <x:v>One pinned 100-task repo snapshot.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="17" t="str">
-        <x:v>OPS-08</x:v>
+        <x:v>OPS-05</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>tau3 Banking</x:v>
+        <x:v>TheAgentCompany</x:v>
       </x:c>
       <x:c r="C27" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D27" s="18" t="n">
-        <x:v>45929</x:v>
+        <x:v>45645</x:v>
       </x:c>
       <x:c r="E27" s="17" t="str">
-        <x:v>2025-Q3</x:v>
+        <x:v>2024-Q4</x:v>
       </x:c>
       <x:c r="F27" s="17" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G27" s="24" t="n">
-        <x:v>0.253</x:v>
+        <x:v>0.24</x:v>
       </x:c>
       <x:c r="H27" s="17" t="str">
-        <x:v>Claude Sonnet 4.5</x:v>
+        <x:v>Launch-paper best system</x:v>
       </x:c>
       <x:c r="I27" s="17" t="str">
-        <x:v>tau3 Banking strict success</x:v>
+        <x:v>Fraction of tasks completed</x:v>
       </x:c>
       <x:c r="J27" s="17" t="str">
-        <x:v>https://taubench.com/leaderboard/</x:v>
+        <x:v>https://arxiv.org/abs/2412.14161</x:v>
       </x:c>
       <x:c r="K27" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Primary-paper baseline.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="17" t="str">
-        <x:v>OPS-08</x:v>
+        <x:v>OPS-05</x:v>
       </x:c>
       <x:c r="B28" s="17" t="str">
-        <x:v>tau3 Banking</x:v>
+        <x:v>TheAgentCompany</x:v>
       </x:c>
       <x:c r="C28" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D28" s="18" t="n">
-        <x:v>46002</x:v>
+        <x:v>45825</x:v>
       </x:c>
       <x:c r="E28" s="17" t="str">
-        <x:v>2025-Q4</x:v>
+        <x:v>2025-Q2</x:v>
       </x:c>
       <x:c r="F28" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G28" s="24" t="n">
-        <x:v>0.322</x:v>
+        <x:v>0.303</x:v>
       </x:c>
       <x:c r="H28" s="17" t="str">
-        <x:v>GPT-5.2</x:v>
+        <x:v>Gemini 2.5 Pro</x:v>
       </x:c>
       <x:c r="I28" s="17" t="str">
-        <x:v>tau3 Banking strict success</x:v>
+        <x:v>Fraction of tasks completed</x:v>
       </x:c>
       <x:c r="J28" s="17" t="str">
-        <x:v>https://taubench.com/leaderboard/</x:v>
+        <x:v>https://the-agent-company.com/</x:v>
       </x:c>
       <x:c r="K28" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Later leaderboard configuration; comparability caveat.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="17" t="str">
-        <x:v>OPS-08</x:v>
+        <x:v>OPS-05</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>tau3 Banking</x:v>
+        <x:v>TheAgentCompany</x:v>
       </x:c>
       <x:c r="C29" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D29" s="18" t="n">
-        <x:v>46086</x:v>
+        <x:v>45901</x:v>
       </x:c>
       <x:c r="E29" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2025-Q3</x:v>
       </x:c>
       <x:c r="F29" s="17" t="n">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G29" s="24" t="n">
-        <x:v>0.394</x:v>
+        <x:v>0.429</x:v>
       </x:c>
       <x:c r="H29" s="17" t="str">
-        <x:v>GPT-5.4</x:v>
+        <x:v>DeepSeek V3.2 + specialized harness</x:v>
       </x:c>
       <x:c r="I29" s="17" t="str">
-        <x:v>tau3 Banking strict success</x:v>
+        <x:v>Fraction of tasks completed</x:v>
       </x:c>
       <x:c r="J29" s="17" t="str">
-        <x:v>https://taubench.com/leaderboard/</x:v>
+        <x:v>https://the-agent-company.com/</x:v>
       </x:c>
       <x:c r="K29" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Community/specialized harness; system-level frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="17" t="str">
-        <x:v>OPS-08</x:v>
+        <x:v>OPS-07</x:v>
       </x:c>
       <x:c r="B30" s="17" t="str">
-        <x:v>tau3 Banking</x:v>
+        <x:v>Finch / FinWorkBench</x:v>
       </x:c>
       <x:c r="C30" s="17" t="str">
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D30" s="18" t="n">
-        <x:v>46143</x:v>
+        <x:v>45974</x:v>
       </x:c>
       <x:c r="E30" s="17" t="str">
-        <x:v>2026-Q2</x:v>
+        <x:v>2025-Q4</x:v>
       </x:c>
       <x:c r="F30" s="17" t="n">
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G30" s="24" t="n">
-        <x:v>0.446</x:v>
+        <x:v>0.384</x:v>
       </x:c>
       <x:c r="H30" s="17" t="str">
-        <x:v>GPT-5.5</x:v>
+        <x:v>GPT-5.1 Pro</x:v>
       </x:c>
       <x:c r="I30" s="17" t="str">
-        <x:v>tau3 Banking strict success</x:v>
+        <x:v>Strict finance-work task pass rate</x:v>
       </x:c>
       <x:c r="J30" s="17" t="str">
-        <x:v>https://taubench.com/leaderboard/</x:v>
+        <x:v>https://aclanthology.org/2026.findings-acl.523/</x:v>
       </x:c>
       <x:c r="K30" s="17" t="str">
-        <x:v>Release-quarter frontier.</x:v>
+        <x:v>Model release-quarter assignment; publication followed in 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -7940,19 +8165,19 @@
         <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D31" s="18" t="n">
-        <x:v>46235</x:v>
+        <x:v>45929</x:v>
       </x:c>
       <x:c r="E31" s="17" t="str">
-        <x:v>2026-Q3</x:v>
+        <x:v>2025-Q3</x:v>
       </x:c>
       <x:c r="F31" s="17" t="n">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G31" s="24" t="n">
-        <x:v>0.552</x:v>
+        <x:v>0.253</x:v>
       </x:c>
       <x:c r="H31" s="17" t="str">
-        <x:v>Qwen 3.8 Max</x:v>
+        <x:v>Claude Sonnet 4.5</x:v>
       </x:c>
       <x:c r="I31" s="17" t="str">
         <x:v>tau3 Banking strict success</x:v>
@@ -7961,56 +8186,56 @@
         <x:v>https://taubench.com/leaderboard/</x:v>
       </x:c>
       <x:c r="K31" s="17" t="str">
-        <x:v>Current quarter frontier.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="17" t="str">
-        <x:v>PER-01</x:v>
+        <x:v>OPS-08</x:v>
       </x:c>
       <x:c r="B32" s="17" t="str">
-        <x:v>MyPCBench</x:v>
+        <x:v>tau3 Banking</x:v>
       </x:c>
       <x:c r="C32" s="17" t="str">
-        <x:v>Personal stewardship transfer</x:v>
+        <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D32" s="18" t="n">
-        <x:v>46058</x:v>
+        <x:v>46002</x:v>
       </x:c>
       <x:c r="E32" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2025-Q4</x:v>
       </x:c>
       <x:c r="F32" s="17" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G32" s="24" t="n">
-        <x:v>0.582</x:v>
+        <x:v>0.322</x:v>
       </x:c>
       <x:c r="H32" s="17" t="str">
-        <x:v>Claude Opus 4.6</x:v>
+        <x:v>GPT-5.2</x:v>
       </x:c>
       <x:c r="I32" s="17" t="str">
-        <x:v>Perfect task success rate</x:v>
+        <x:v>tau3 Banking strict success</x:v>
       </x:c>
       <x:c r="J32" s="17" t="str">
-        <x:v>https://mypcbench.com/</x:v>
+        <x:v>https://taubench.com/leaderboard/</x:v>
       </x:c>
       <x:c r="K32" s="17" t="str">
-        <x:v>Current published frontier; newer models may be missing.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="17" t="str">
-        <x:v>PER-02</x:v>
+        <x:v>OPS-08</x:v>
       </x:c>
       <x:c r="B33" s="17" t="str">
-        <x:v>pi-Bench</x:v>
+        <x:v>tau3 Banking</x:v>
       </x:c>
       <x:c r="C33" s="17" t="str">
-        <x:v>Personal stewardship transfer</x:v>
+        <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D33" s="18" t="n">
-        <x:v>46058</x:v>
+        <x:v>46086</x:v>
       </x:c>
       <x:c r="E33" s="17" t="str">
         <x:v>2026-Q1</x:v>
@@ -8019,33 +8244,33 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="G33" s="24" t="n">
-        <x:v>0.676</x:v>
+        <x:v>0.394</x:v>
       </x:c>
       <x:c r="H33" s="17" t="str">
-        <x:v>Claude Opus 4.6</x:v>
+        <x:v>GPT-5.4</x:v>
       </x:c>
       <x:c r="I33" s="17" t="str">
-        <x:v>Completeness checklist score</x:v>
+        <x:v>tau3 Banking strict success</x:v>
       </x:c>
       <x:c r="J33" s="17" t="str">
-        <x:v>https://arxiv.org/html/2605.14678v3</x:v>
+        <x:v>https://taubench.com/leaderboard/</x:v>
       </x:c>
       <x:c r="K33" s="17" t="str">
-        <x:v>One comparable frontier point.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="17" t="str">
-        <x:v>PER-03</x:v>
+        <x:v>OPS-08</x:v>
       </x:c>
       <x:c r="B34" s="17" t="str">
-        <x:v>ClawBench</x:v>
+        <x:v>tau3 Banking</x:v>
       </x:c>
       <x:c r="C34" s="17" t="str">
-        <x:v>Personal stewardship transfer</x:v>
+        <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D34" s="18" t="n">
-        <x:v>46174</x:v>
+        <x:v>46143</x:v>
       </x:c>
       <x:c r="E34" s="17" t="str">
         <x:v>2026-Q2</x:v>
@@ -8054,263 +8279,403 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="G34" s="24" t="n">
-        <x:v>0.333</x:v>
+        <x:v>0.446</x:v>
       </x:c>
       <x:c r="H34" s="17" t="str">
-        <x:v>Current top system</x:v>
+        <x:v>GPT-5.5</x:v>
       </x:c>
       <x:c r="I34" s="17" t="str">
-        <x:v>Standardized ClawBench score</x:v>
+        <x:v>tau3 Banking strict success</x:v>
       </x:c>
       <x:c r="J34" s="17" t="str">
-        <x:v>https://github.com/TIGER-AI-Lab/ClawBench</x:v>
+        <x:v>https://taubench.com/leaderboard/</x:v>
       </x:c>
       <x:c r="K34" s="17" t="str">
-        <x:v>One public frontier point; pin repository version.</x:v>
+        <x:v>Release-quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="17" t="str">
-        <x:v>PER-04</x:v>
+        <x:v>OPS-08</x:v>
       </x:c>
       <x:c r="B35" s="17" t="str">
-        <x:v>AssistantBench</x:v>
+        <x:v>tau3 Banking</x:v>
       </x:c>
       <x:c r="C35" s="17" t="str">
-        <x:v>Personal stewardship transfer</x:v>
+        <x:v>Operational execution</x:v>
       </x:c>
       <x:c r="D35" s="18" t="n">
-        <x:v>45545</x:v>
+        <x:v>46235</x:v>
       </x:c>
       <x:c r="E35" s="17" t="str">
-        <x:v>2024-Q3</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="F35" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G35" s="24" t="n">
-        <x:v>0.252</x:v>
+        <x:v>0.552</x:v>
       </x:c>
       <x:c r="H35" s="17" t="str">
-        <x:v>Launch-paper top system</x:v>
+        <x:v>Qwen 3.8 Max</x:v>
       </x:c>
       <x:c r="I35" s="17" t="str">
-        <x:v>Assistant task accuracy</x:v>
+        <x:v>tau3 Banking strict success</x:v>
       </x:c>
       <x:c r="J35" s="17" t="str">
-        <x:v>https://assistantbench.github.io/</x:v>
+        <x:v>https://taubench.com/leaderboard/</x:v>
       </x:c>
       <x:c r="K35" s="17" t="str">
-        <x:v>Original benchmark configuration.</x:v>
+        <x:v>Current quarter frontier.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="17" t="str">
-        <x:v>PER-04</x:v>
+        <x:v>PER-01</x:v>
       </x:c>
       <x:c r="B36" s="17" t="str">
-        <x:v>AssistantBench</x:v>
+        <x:v>MyPCBench</x:v>
       </x:c>
       <x:c r="C36" s="17" t="str">
         <x:v>Personal stewardship transfer</x:v>
       </x:c>
       <x:c r="D36" s="18" t="n">
-        <x:v>45876</x:v>
+        <x:v>46058</x:v>
       </x:c>
       <x:c r="E36" s="17" t="str">
-        <x:v>2025-Q3</x:v>
+        <x:v>2026-Q1</x:v>
       </x:c>
       <x:c r="F36" s="17" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G36" s="24" t="n">
-        <x:v>0.367</x:v>
+        <x:v>0.582</x:v>
       </x:c>
       <x:c r="H36" s="17" t="str">
-        <x:v>GPT-5</x:v>
+        <x:v>Claude Opus 4.6</x:v>
       </x:c>
       <x:c r="I36" s="17" t="str">
-        <x:v>Assistant task accuracy</x:v>
+        <x:v>Perfect task success rate</x:v>
       </x:c>
       <x:c r="J36" s="17" t="str">
-        <x:v>https://hal.cs.princeton.edu/assistantbench</x:v>
+        <x:v>https://mypcbench.com/</x:v>
       </x:c>
       <x:c r="K36" s="17" t="str">
-        <x:v>Updated HAL leaderboard/configuration; system-level trend only.</x:v>
+        <x:v>Current published frontier; newer models may be missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="17" t="str">
-        <x:v>VAL-02</x:v>
+        <x:v>PER-02</x:v>
       </x:c>
       <x:c r="B37" s="17" t="str">
-        <x:v>Remote Labor Index</x:v>
+        <x:v>pi-Bench</x:v>
       </x:c>
       <x:c r="C37" s="17" t="str">
-        <x:v>Economic value &amp; governance</x:v>
+        <x:v>Personal stewardship transfer</x:v>
       </x:c>
       <x:c r="D37" s="18" t="n">
-        <x:v>45929</x:v>
+        <x:v>46058</x:v>
       </x:c>
       <x:c r="E37" s="17" t="str">
-        <x:v>2025-Q3</x:v>
+        <x:v>2026-Q1</x:v>
       </x:c>
       <x:c r="F37" s="17" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G37" s="24" t="n">
-        <x:v>0.0208</x:v>
+        <x:v>0.676</x:v>
       </x:c>
       <x:c r="H37" s="17" t="str">
-        <x:v>Claude Sonnet 4.5</x:v>
+        <x:v>Claude Opus 4.6</x:v>
       </x:c>
       <x:c r="I37" s="17" t="str">
-        <x:v>Strict end-to-end automation rate</x:v>
+        <x:v>Completeness checklist score</x:v>
       </x:c>
       <x:c r="J37" s="17" t="str">
-        <x:v>https://www.remotelabor.ai/</x:v>
+        <x:v>https://arxiv.org/html/2605.14678v3</x:v>
       </x:c>
       <x:c r="K37" s="17" t="str">
-        <x:v>Quarter frontier.</x:v>
+        <x:v>One comparable frontier point.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="17" t="str">
-        <x:v>VAL-02</x:v>
+        <x:v>PER-03</x:v>
       </x:c>
       <x:c r="B38" s="17" t="str">
-        <x:v>Remote Labor Index</x:v>
+        <x:v>ClawBench</x:v>
       </x:c>
       <x:c r="C38" s="17" t="str">
-        <x:v>Economic value &amp; governance</x:v>
+        <x:v>Personal stewardship transfer</x:v>
       </x:c>
       <x:c r="D38" s="18" t="n">
-        <x:v>45985</x:v>
+        <x:v>46174</x:v>
       </x:c>
       <x:c r="E38" s="17" t="str">
-        <x:v>2025-Q4</x:v>
+        <x:v>2026-Q2</x:v>
       </x:c>
       <x:c r="F38" s="17" t="n">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G38" s="24" t="n">
-        <x:v>0.0375</x:v>
+        <x:v>0.333</x:v>
       </x:c>
       <x:c r="H38" s="17" t="str">
-        <x:v>Claude Opus 4.5</x:v>
+        <x:v>Current top system</x:v>
       </x:c>
       <x:c r="I38" s="17" t="str">
-        <x:v>Strict end-to-end automation rate</x:v>
+        <x:v>Standardized ClawBench score</x:v>
       </x:c>
       <x:c r="J38" s="17" t="str">
-        <x:v>https://www.remotelabor.ai/</x:v>
+        <x:v>https://github.com/TIGER-AI-Lab/ClawBench</x:v>
       </x:c>
       <x:c r="K38" s="17" t="str">
-        <x:v>Quarter frontier.</x:v>
+        <x:v>One public frontier point; pin repository version.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="17" t="str">
-        <x:v>VAL-02</x:v>
+        <x:v>PER-04</x:v>
       </x:c>
       <x:c r="B39" s="17" t="str">
-        <x:v>Remote Labor Index</x:v>
+        <x:v>AssistantBench</x:v>
       </x:c>
       <x:c r="C39" s="17" t="str">
-        <x:v>Economic value &amp; governance</x:v>
+        <x:v>Personal stewardship transfer</x:v>
       </x:c>
       <x:c r="D39" s="18" t="n">
-        <x:v>46058</x:v>
+        <x:v>45545</x:v>
       </x:c>
       <x:c r="E39" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2024-Q3</x:v>
       </x:c>
       <x:c r="F39" s="17" t="n">
-        <x:v>9</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G39" s="24" t="n">
-        <x:v>0.0417</x:v>
+        <x:v>0.252</x:v>
       </x:c>
       <x:c r="H39" s="17" t="str">
-        <x:v>Claude Opus 4.6</x:v>
+        <x:v>Launch-paper top system</x:v>
       </x:c>
       <x:c r="I39" s="17" t="str">
-        <x:v>Strict end-to-end automation rate</x:v>
+        <x:v>Assistant task accuracy</x:v>
       </x:c>
       <x:c r="J39" s="17" t="str">
-        <x:v>https://www.remotelabor.ai/</x:v>
+        <x:v>https://assistantbench.github.io/</x:v>
       </x:c>
       <x:c r="K39" s="17" t="str">
-        <x:v>Quarter frontier.</x:v>
+        <x:v>Original benchmark configuration.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="17" t="str">
-        <x:v>VAL-02</x:v>
+        <x:v>PER-04</x:v>
       </x:c>
       <x:c r="B40" s="17" t="str">
-        <x:v>Remote Labor Index</x:v>
+        <x:v>AssistantBench</x:v>
       </x:c>
       <x:c r="C40" s="17" t="str">
-        <x:v>Economic value &amp; governance</x:v>
+        <x:v>Personal stewardship transfer</x:v>
       </x:c>
       <x:c r="D40" s="18" t="n">
-        <x:v>46182</x:v>
+        <x:v>45876</x:v>
       </x:c>
       <x:c r="E40" s="17" t="str">
-        <x:v>2026-Q2</x:v>
+        <x:v>2025-Q3</x:v>
       </x:c>
       <x:c r="F40" s="17" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G40" s="24" t="n">
-        <x:v>0.158</x:v>
+        <x:v>0.367</x:v>
       </x:c>
       <x:c r="H40" s="17" t="str">
-        <x:v>Claude Fable 5</x:v>
+        <x:v>GPT-5</x:v>
       </x:c>
       <x:c r="I40" s="17" t="str">
-        <x:v>Strict end-to-end automation rate</x:v>
+        <x:v>Assistant task accuracy</x:v>
       </x:c>
       <x:c r="J40" s="17" t="str">
-        <x:v>https://www.remotelabor.ai/</x:v>
+        <x:v>https://hal.cs.princeton.edu/assistantbench</x:v>
       </x:c>
       <x:c r="K40" s="17" t="str">
-        <x:v>Current frontier; large quarter jump merits caution.</x:v>
+        <x:v>Updated HAL leaderboard/configuration; system-level trend only.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="17" t="str">
-        <x:v>VAL-04</x:v>
+        <x:v>VAL-02</x:v>
       </x:c>
       <x:c r="B41" s="17" t="str">
-        <x:v>Claw-Eval</x:v>
+        <x:v>Remote Labor Index</x:v>
       </x:c>
       <x:c r="C41" s="17" t="str">
         <x:v>Economic value &amp; governance</x:v>
       </x:c>
       <x:c r="D41" s="18" t="n">
+        <x:v>45929</x:v>
+      </x:c>
+      <x:c r="E41" s="17" t="str">
+        <x:v>2025-Q3</x:v>
+      </x:c>
+      <x:c r="F41" s="17" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G41" s="24" t="n">
+        <x:v>0.0208</x:v>
+      </x:c>
+      <x:c r="H41" s="17" t="str">
+        <x:v>Claude Sonnet 4.5</x:v>
+      </x:c>
+      <x:c r="I41" s="17" t="str">
+        <x:v>Strict end-to-end automation rate</x:v>
+      </x:c>
+      <x:c r="J41" s="17" t="str">
+        <x:v>https://www.remotelabor.ai/</x:v>
+      </x:c>
+      <x:c r="K41" s="17" t="str">
+        <x:v>Quarter frontier.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="17" t="str">
+        <x:v>VAL-02</x:v>
+      </x:c>
+      <x:c r="B42" s="17" t="str">
+        <x:v>Remote Labor Index</x:v>
+      </x:c>
+      <x:c r="C42" s="17" t="str">
+        <x:v>Economic value &amp; governance</x:v>
+      </x:c>
+      <x:c r="D42" s="18" t="n">
+        <x:v>45985</x:v>
+      </x:c>
+      <x:c r="E42" s="17" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="F42" s="17" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G42" s="24" t="n">
+        <x:v>0.0375</x:v>
+      </x:c>
+      <x:c r="H42" s="17" t="str">
+        <x:v>Claude Opus 4.5</x:v>
+      </x:c>
+      <x:c r="I42" s="17" t="str">
+        <x:v>Strict end-to-end automation rate</x:v>
+      </x:c>
+      <x:c r="J42" s="17" t="str">
+        <x:v>https://www.remotelabor.ai/</x:v>
+      </x:c>
+      <x:c r="K42" s="17" t="str">
+        <x:v>Quarter frontier.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="17" t="str">
+        <x:v>VAL-02</x:v>
+      </x:c>
+      <x:c r="B43" s="17" t="str">
+        <x:v>Remote Labor Index</x:v>
+      </x:c>
+      <x:c r="C43" s="17" t="str">
+        <x:v>Economic value &amp; governance</x:v>
+      </x:c>
+      <x:c r="D43" s="18" t="n">
         <x:v>46058</x:v>
       </x:c>
-      <x:c r="E41" s="17" t="str">
+      <x:c r="E43" s="17" t="str">
         <x:v>2026-Q1</x:v>
       </x:c>
-      <x:c r="F41" s="17" t="n">
+      <x:c r="F43" s="17" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="G41" s="24" t="n">
+      <x:c r="G43" s="24" t="n">
+        <x:v>0.0417</x:v>
+      </x:c>
+      <x:c r="H43" s="17" t="str">
+        <x:v>Claude Opus 4.6</x:v>
+      </x:c>
+      <x:c r="I43" s="17" t="str">
+        <x:v>Strict end-to-end automation rate</x:v>
+      </x:c>
+      <x:c r="J43" s="17" t="str">
+        <x:v>https://www.remotelabor.ai/</x:v>
+      </x:c>
+      <x:c r="K43" s="17" t="str">
+        <x:v>Quarter frontier.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="17" t="str">
+        <x:v>VAL-02</x:v>
+      </x:c>
+      <x:c r="B44" s="17" t="str">
+        <x:v>Remote Labor Index</x:v>
+      </x:c>
+      <x:c r="C44" s="17" t="str">
+        <x:v>Economic value &amp; governance</x:v>
+      </x:c>
+      <x:c r="D44" s="18" t="n">
+        <x:v>46182</x:v>
+      </x:c>
+      <x:c r="E44" s="17" t="str">
+        <x:v>2026-Q2</x:v>
+      </x:c>
+      <x:c r="F44" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G44" s="24" t="n">
+        <x:v>0.158</x:v>
+      </x:c>
+      <x:c r="H44" s="17" t="str">
+        <x:v>Claude Fable 5</x:v>
+      </x:c>
+      <x:c r="I44" s="17" t="str">
+        <x:v>Strict end-to-end automation rate</x:v>
+      </x:c>
+      <x:c r="J44" s="17" t="str">
+        <x:v>https://www.remotelabor.ai/</x:v>
+      </x:c>
+      <x:c r="K44" s="17" t="str">
+        <x:v>Current frontier; large quarter jump merits caution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="17" t="str">
+        <x:v>VAL-04</x:v>
+      </x:c>
+      <x:c r="B45" s="17" t="str">
+        <x:v>Claw-Eval</x:v>
+      </x:c>
+      <x:c r="C45" s="17" t="str">
+        <x:v>Economic value &amp; governance</x:v>
+      </x:c>
+      <x:c r="D45" s="18" t="n">
+        <x:v>46058</x:v>
+      </x:c>
+      <x:c r="E45" s="17" t="str">
+        <x:v>2026-Q1</x:v>
+      </x:c>
+      <x:c r="F45" s="17" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G45" s="24" t="n">
         <x:v>0.704</x:v>
       </x:c>
-      <x:c r="H41" s="17" t="str">
+      <x:c r="H45" s="17" t="str">
         <x:v>Claude Opus 4.6</x:v>
       </x:c>
-      <x:c r="I41" s="17" t="str">
+      <x:c r="I45" s="17" t="str">
         <x:v>Pass^3 governed-agent score</x:v>
       </x:c>
-      <x:c r="J41" s="17" t="str">
+      <x:c r="J45" s="17" t="str">
         <x:v>https://github.com/claw-eval/claw-eval</x:v>
       </x:c>
-      <x:c r="K41" s="17" t="str">
+      <x:c r="K45" s="17" t="str">
         <x:v>One current frontier point.</x:v>
       </x:c>
     </x:row>
@@ -8320,18 +8685,18 @@
     <x:mergeCell ref="A3:K3"/>
   </x:mergeCells>
   <x:dataValidations count="2">
-    <x:dataValidation operator="between" sqref="F6:F41">
+    <x:dataValidation operator="between" sqref="F6:F45">
       <x:formula1>1</x:formula1>
       <x:formula2>20</x:formula2>
     </x:dataValidation>
-    <x:dataValidation type="decimal" operator="between" sqref="G6:G41">
+    <x:dataValidation type="decimal" operator="between" sqref="G6:G45">
       <x:formula1>0</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb65dcf679a924ac1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re04d5d05bbb94ddb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8537,13 +8902,13 @@
         <x:v>YC-Bench</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>One-year startup final funds</x:v>
+        <x:v>Frontier mean final funds / $1M published substantial-profit threshold</x:v>
       </x:c>
       <x:c r="E8" s="17" t="str">
-        <x:v>Ungraded until a defensible success ceiling or target is published</x:v>
+        <x:v>Cap at 100%; provisional target-normalized score because no human/oracle result is published</x:v>
       </x:c>
       <x:c r="F8" s="17" t="str">
-        <x:v>Ungraded</x:v>
+        <x:v>Graded</x:v>
       </x:c>
       <x:c r="G8" s="17" t="str">
         <x:v>2026-Q2</x:v>
@@ -8552,10 +8917,10 @@
         <x:v>https://arxiv.org/abs/2604.01212</x:v>
       </x:c>
       <x:c r="I8" s="17" t="str">
-        <x:v>Dollar outcomes cannot be converted to completion percentages without an anchor.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+        <x:v>The frontier exceeds the paper's 5×-capital threshold, so this score is saturated and needs a harder future anchor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>DES-04</x:v>
       </x:c>
@@ -8566,22 +8931,22 @@
         <x:v>Business Arena</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>30-day seller final worth</x:v>
+        <x:v>Best-model mean final worth / $436,195 expert-strategy final worth</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
-        <x:v>Ungraded until the human/reference strategy value is published</x:v>
+        <x:v>Cap at 100%; fixed expert strategy uses agent-visible information in the same world</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>Ungraded</x:v>
+        <x:v>Graded</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
-        <x:v>2026-Q1</x:v>
+        <x:v>2026-Q3</x:v>
       </x:c>
       <x:c r="H9" s="17" t="str">
-        <x:v>https://github.com/Accio-org/BusinessArena</x:v>
+        <x:v>https://arxiv.org/abs/2608.08621</x:v>
       </x:c>
       <x:c r="I9" s="17" t="str">
-        <x:v>Reference strategies exist, but no stable saturation denominator was sourced.</x:v>
+        <x:v>Ten-run model mean divided by the strongest published expert-designed strategy outcome.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -8613,7 +8978,7 @@
         <x:v>132-month CFO simulator; current point has limited-run uncertainty.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>DES-06</x:v>
       </x:c>
@@ -8624,13 +8989,13 @@
         <x:v>RetailBench</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str">
-        <x:v>Long-horizon retail operations score</x:v>
+        <x:v>Best LLM final net worth / $131,510.42 oracle final net worth</x:v>
       </x:c>
       <x:c r="E11" s="17" t="str">
-        <x:v>Ungraded until a current normalized frontier result is sourceable</x:v>
+        <x:v>Cap at 100%; privileged oracle is a ceiling-like reference, not a human-equivalent baseline</x:v>
       </x:c>
       <x:c r="F11" s="17" t="str">
-        <x:v>Ungraded</x:v>
+        <x:v>Graded</x:v>
       </x:c>
       <x:c r="G11" s="17" t="str">
         <x:v>2026-Q1</x:v>
@@ -8639,10 +9004,10 @@
         <x:v>https://arxiv.org/abs/2603.16453</x:v>
       </x:c>
       <x:c r="I11" s="17" t="str">
-        <x:v>Cataloged for future observations.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>Uses the v3 selected-run table; result is framework-selected and not a repeated-run mean.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A12" s="17" t="str">
         <x:v>DES-07</x:v>
       </x:c>
@@ -8653,13 +9018,13 @@
         <x:v>MerchantBench</x:v>
       </x:c>
       <x:c r="D12" s="17" t="str">
-        <x:v>365-day ecommerce operating score</x:v>
+        <x:v>Best LLM mean final net assets / human-participant mean</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:v>Ungraded until a normalized frontier result is published</x:v>
+        <x:v>Use the authors' reported 27.3% human-relative ratio</x:v>
       </x:c>
       <x:c r="F12" s="17" t="str">
-        <x:v>Ungraded</x:v>
+        <x:v>Graded</x:v>
       </x:c>
       <x:c r="G12" s="17" t="str">
         <x:v>2026-Q3</x:v>
@@ -8668,7 +9033,7 @@
         <x:v>https://arxiv.org/abs/2607.28956</x:v>
       </x:c>
       <x:c r="I12" s="17" t="str">
-        <x:v>New benchmark; cataloged without inventing a launch score.</x:v>
+        <x:v>Three runs per model-framework pairing; human reference is three non-expert participants.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -9147,7 +9512,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5e01cd075ec4ac4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0286647e1cca4d78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9406,13 +9771,13 @@
         <x:v>Latest depth</x:v>
       </x:c>
       <x:c r="N5" s="13" t="str">
-        <x:v>Recent velocity</x:v>
+        <x:v>Recent gap velocity</x:v>
       </x:c>
       <x:c r="O5" s="13" t="str">
-        <x:v>Prior velocity</x:v>
+        <x:v>Prior gap velocity</x:v>
       </x:c>
       <x:c r="P5" s="13" t="str">
-        <x:v>Acceleration</x:v>
+        <x:v>Gap acceleration</x:v>
       </x:c>
       <x:c r="Q5" s="13" t="str">
         <x:v>Projection basis</x:v>
@@ -9466,15 +9831,15 @@
         <x:v>0.17749</x:v>
       </x:c>
       <x:c r="K6" s="25" t="n">
-        <x:f>IF(H6="","",-LN(1-H6)/LN(2))</x:f>
+        <x:f>IF(H6="","",IF(H6&gt;=1,30,-LN(1-H6)/LN(2)))</x:f>
         <x:v>0.19638168387795835</x:v>
       </x:c>
       <x:c r="L6" s="25" t="n">
-        <x:f>IF(I6="","",-LN(1-I6)/LN(2))</x:f>
+        <x:f>IF(I6="","",IF(I6&gt;=1,30,-LN(1-I6)/LN(2)))</x:f>
         <x:v>0.27508673226655406</x:v>
       </x:c>
       <x:c r="M6" s="25" t="n">
-        <x:f>IF(J6="","",-LN(1-J6)/LN(2))</x:f>
+        <x:f>IF(J6="","",IF(J6&gt;=1,30,-LN(1-J6)/LN(2)))</x:f>
         <x:v>0.28189487578087197</x:v>
       </x:c>
       <x:c r="N6" s="25" t="n">
@@ -9543,14 +9908,14 @@
         <x:v>0.010067435</x:v>
       </x:c>
       <x:c r="K7" s="25" t="str">
-        <x:f>IF(H7="","",-LN(1-H7)/LN(2))</x:f>
+        <x:f>IF(H7="","",IF(H7&gt;=1,30,-LN(1-H7)/LN(2)))</x:f>
       </x:c>
       <x:c r="L7" s="25" t="n">
-        <x:f>IF(I7="","",-LN(1-I7)/LN(2))</x:f>
+        <x:f>IF(I7="","",IF(I7&gt;=1,30,-LN(1-I7)/LN(2)))</x:f>
         <x:v>0.008306298103420784</x:v>
       </x:c>
       <x:c r="M7" s="25" t="n">
-        <x:f>IF(J7="","",-LN(1-J7)/LN(2))</x:f>
+        <x:f>IF(J7="","",IF(J7&gt;=1,30,-LN(1-J7)/LN(2)))</x:f>
         <x:v>0.01459784389075154</x:v>
       </x:c>
       <x:c r="N7" s="25" t="n">
@@ -9594,7 +9959,7 @@
       </x:c>
       <x:c r="D8" s="17" t="n">
         <x:f>COUNTIF('Observations'!$A$6:$A$500,A8)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E8" s="17" t="str">
         <x:f>IF(D8&lt;3,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A8,'Observations'!$F$6:$F$500,"&lt;"&amp;F8))</x:f>
@@ -9602,8 +9967,9 @@
       <x:c r="F8" s="17" t="str">
         <x:f>IF(D8&lt;2,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A8,'Observations'!$F$6:$F$500,"&lt;"&amp;G8))</x:f>
       </x:c>
-      <x:c r="G8" s="17" t="str">
+      <x:c r="G8" s="17" t="n">
         <x:f>IF(D8=0,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A8))</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
         <x:f>IF(E8="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A8,'Observations'!$F$6:$F$500,E8))</x:f>
@@ -9611,17 +9977,19 @@
       <x:c r="I8" s="24" t="str">
         <x:f>IF(F8="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A8,'Observations'!$F$6:$F$500,F8))</x:f>
       </x:c>
-      <x:c r="J8" s="24" t="str">
+      <x:c r="J8" s="24" t="n">
         <x:f>IF(G8="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A8,'Observations'!$F$6:$F$500,G8))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K8" s="25" t="str">
-        <x:f>IF(H8="","",-LN(1-H8)/LN(2))</x:f>
+        <x:f>IF(H8="","",IF(H8&gt;=1,30,-LN(1-H8)/LN(2)))</x:f>
       </x:c>
       <x:c r="L8" s="25" t="str">
-        <x:f>IF(I8="","",-LN(1-I8)/LN(2))</x:f>
-      </x:c>
-      <x:c r="M8" s="25" t="str">
-        <x:f>IF(J8="","",-LN(1-J8)/LN(2))</x:f>
+        <x:f>IF(I8="","",IF(I8&gt;=1,30,-LN(1-I8)/LN(2)))</x:f>
+      </x:c>
+      <x:c r="M8" s="25" t="n">
+        <x:f>IF(J8="","",IF(J8&gt;=1,30,-LN(1-J8)/LN(2)))</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="N8" s="25" t="n">
         <x:f>IF(D8&lt;2,0,(M8-L8)/(G8-F8))</x:f>
@@ -9637,17 +10005,19 @@
       </x:c>
       <x:c r="Q8" s="17" t="str">
         <x:f>IF(D8=0,"Ungraded — no normalized observation",IF(D8=1,"Flat — one observation",IF(D8=2,"Constant velocity — two observations","Velocity + acceleration — latest three observations")))</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
-      </x:c>
-      <x:c r="R8" s="24" t="str">
+        <x:v>Flat — one observation</x:v>
+      </x:c>
+      <x:c r="R8" s="24" t="n">
         <x:f>IF(D8=0,"",J8)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="S8" s="17" t="str">
         <x:f>IF(R8="","N/A",IF(R8&gt;='Methodology'!$G$7,"A",IF(R8&gt;='Methodology'!$G$8,"B",IF(R8&gt;='Methodology'!$G$9,"C",IF(R8&gt;='Methodology'!$G$10,"D","F")))))</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="T8" s="26" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="T8" s="26" t="n">
         <x:f>IF(R8="","",IF(R8&gt;='Methodology'!$G$7,'Methodology'!$H$7,IF(R8&gt;='Methodology'!$G$8,'Methodology'!$H$8,IF(R8&gt;='Methodology'!$G$9,'Methodology'!$H$9,IF(R8&gt;='Methodology'!$G$10,'Methodology'!$H$10,'Methodology'!$H$11)))))</x:f>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -9662,7 +10032,7 @@
       </x:c>
       <x:c r="D9" s="17" t="n">
         <x:f>COUNTIF('Observations'!$A$6:$A$500,A9)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
         <x:f>IF(D9&lt;3,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A9,'Observations'!$F$6:$F$500,"&lt;"&amp;F9))</x:f>
@@ -9670,8 +10040,9 @@
       <x:c r="F9" s="17" t="str">
         <x:f>IF(D9&lt;2,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A9,'Observations'!$F$6:$F$500,"&lt;"&amp;G9))</x:f>
       </x:c>
-      <x:c r="G9" s="17" t="str">
+      <x:c r="G9" s="17" t="n">
         <x:f>IF(D9=0,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A9))</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
         <x:f>IF(E9="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A9,'Observations'!$F$6:$F$500,E9))</x:f>
@@ -9679,17 +10050,19 @@
       <x:c r="I9" s="24" t="str">
         <x:f>IF(F9="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A9,'Observations'!$F$6:$F$500,F9))</x:f>
       </x:c>
-      <x:c r="J9" s="24" t="str">
+      <x:c r="J9" s="24" t="n">
         <x:f>IF(G9="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A9,'Observations'!$F$6:$F$500,G9))</x:f>
+        <x:v>0.4321186625247882</x:v>
       </x:c>
       <x:c r="K9" s="25" t="str">
-        <x:f>IF(H9="","",-LN(1-H9)/LN(2))</x:f>
+        <x:f>IF(H9="","",IF(H9&gt;=1,30,-LN(1-H9)/LN(2)))</x:f>
       </x:c>
       <x:c r="L9" s="25" t="str">
-        <x:f>IF(I9="","",-LN(1-I9)/LN(2))</x:f>
-      </x:c>
-      <x:c r="M9" s="25" t="str">
-        <x:f>IF(J9="","",-LN(1-J9)/LN(2))</x:f>
+        <x:f>IF(I9="","",IF(I9&gt;=1,30,-LN(1-I9)/LN(2)))</x:f>
+      </x:c>
+      <x:c r="M9" s="25" t="n">
+        <x:f>IF(J9="","",IF(J9&gt;=1,30,-LN(1-J9)/LN(2)))</x:f>
+        <x:v>0.8163385942433947</x:v>
       </x:c>
       <x:c r="N9" s="25" t="n">
         <x:f>IF(D9&lt;2,0,(M9-L9)/(G9-F9))</x:f>
@@ -9705,17 +10078,19 @@
       </x:c>
       <x:c r="Q9" s="17" t="str">
         <x:f>IF(D9=0,"Ungraded — no normalized observation",IF(D9=1,"Flat — one observation",IF(D9=2,"Constant velocity — two observations","Velocity + acceleration — latest three observations")))</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
-      </x:c>
-      <x:c r="R9" s="24" t="str">
+        <x:v>Flat — one observation</x:v>
+      </x:c>
+      <x:c r="R9" s="24" t="n">
         <x:f>IF(D9=0,"",J9)</x:f>
+        <x:v>0.4321186625247882</x:v>
       </x:c>
       <x:c r="S9" s="17" t="str">
         <x:f>IF(R9="","N/A",IF(R9&gt;='Methodology'!$G$7,"A",IF(R9&gt;='Methodology'!$G$8,"B",IF(R9&gt;='Methodology'!$G$9,"C",IF(R9&gt;='Methodology'!$G$10,"D","F")))))</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="T9" s="26" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="T9" s="26" t="n">
         <x:f>IF(R9="","",IF(R9&gt;='Methodology'!$G$7,'Methodology'!$H$7,IF(R9&gt;='Methodology'!$G$8,'Methodology'!$H$8,IF(R9&gt;='Methodology'!$G$9,'Methodology'!$H$9,IF(R9&gt;='Methodology'!$G$10,'Methodology'!$H$10,'Methodology'!$H$11)))))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -9753,13 +10128,13 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="K10" s="25" t="str">
-        <x:f>IF(H10="","",-LN(1-H10)/LN(2))</x:f>
+        <x:f>IF(H10="","",IF(H10&gt;=1,30,-LN(1-H10)/LN(2)))</x:f>
       </x:c>
       <x:c r="L10" s="25" t="str">
-        <x:f>IF(I10="","",-LN(1-I10)/LN(2))</x:f>
+        <x:f>IF(I10="","",IF(I10&gt;=1,30,-LN(1-I10)/LN(2)))</x:f>
       </x:c>
       <x:c r="M10" s="25" t="n">
-        <x:f>IF(J10="","",-LN(1-J10)/LN(2))</x:f>
+        <x:f>IF(J10="","",IF(J10&gt;=1,30,-LN(1-J10)/LN(2)))</x:f>
         <x:v>2.3219280948873626</x:v>
       </x:c>
       <x:c r="N10" s="25" t="n">
@@ -9803,7 +10178,7 @@
       </x:c>
       <x:c r="D11" s="17" t="n">
         <x:f>COUNTIF('Observations'!$A$6:$A$500,A11)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E11" s="17" t="str">
         <x:f>IF(D11&lt;3,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A11,'Observations'!$F$6:$F$500,"&lt;"&amp;F11))</x:f>
@@ -9811,8 +10186,9 @@
       <x:c r="F11" s="17" t="str">
         <x:f>IF(D11&lt;2,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A11,'Observations'!$F$6:$F$500,"&lt;"&amp;G11))</x:f>
       </x:c>
-      <x:c r="G11" s="17" t="str">
+      <x:c r="G11" s="17" t="n">
         <x:f>IF(D11=0,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A11))</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
         <x:f>IF(E11="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A11,'Observations'!$F$6:$F$500,E11))</x:f>
@@ -9820,17 +10196,19 @@
       <x:c r="I11" s="24" t="str">
         <x:f>IF(F11="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A11,'Observations'!$F$6:$F$500,F11))</x:f>
       </x:c>
-      <x:c r="J11" s="24" t="str">
+      <x:c r="J11" s="24" t="n">
         <x:f>IF(G11="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A11,'Observations'!$F$6:$F$500,G11))</x:f>
+        <x:v>0.18516388283148968</x:v>
       </x:c>
       <x:c r="K11" s="25" t="str">
-        <x:f>IF(H11="","",-LN(1-H11)/LN(2))</x:f>
+        <x:f>IF(H11="","",IF(H11&gt;=1,30,-LN(1-H11)/LN(2)))</x:f>
       </x:c>
       <x:c r="L11" s="25" t="str">
-        <x:f>IF(I11="","",-LN(1-I11)/LN(2))</x:f>
-      </x:c>
-      <x:c r="M11" s="25" t="str">
-        <x:f>IF(J11="","",-LN(1-J11)/LN(2))</x:f>
+        <x:f>IF(I11="","",IF(I11&gt;=1,30,-LN(1-I11)/LN(2)))</x:f>
+      </x:c>
+      <x:c r="M11" s="25" t="n">
+        <x:f>IF(J11="","",IF(J11&gt;=1,30,-LN(1-J11)/LN(2)))</x:f>
+        <x:v>0.29541816649188574</x:v>
       </x:c>
       <x:c r="N11" s="25" t="n">
         <x:f>IF(D11&lt;2,0,(M11-L11)/(G11-F11))</x:f>
@@ -9846,17 +10224,19 @@
       </x:c>
       <x:c r="Q11" s="17" t="str">
         <x:f>IF(D11=0,"Ungraded — no normalized observation",IF(D11=1,"Flat — one observation",IF(D11=2,"Constant velocity — two observations","Velocity + acceleration — latest three observations")))</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
-      </x:c>
-      <x:c r="R11" s="24" t="str">
+        <x:v>Flat — one observation</x:v>
+      </x:c>
+      <x:c r="R11" s="24" t="n">
         <x:f>IF(D11=0,"",J11)</x:f>
+        <x:v>0.18516388283148968</x:v>
       </x:c>
       <x:c r="S11" s="17" t="str">
         <x:f>IF(R11="","N/A",IF(R11&gt;='Methodology'!$G$7,"A",IF(R11&gt;='Methodology'!$G$8,"B",IF(R11&gt;='Methodology'!$G$9,"C",IF(R11&gt;='Methodology'!$G$10,"D","F")))))</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="T11" s="26" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="T11" s="26" t="n">
         <x:f>IF(R11="","",IF(R11&gt;='Methodology'!$G$7,'Methodology'!$H$7,IF(R11&gt;='Methodology'!$G$8,'Methodology'!$H$8,IF(R11&gt;='Methodology'!$G$9,'Methodology'!$H$9,IF(R11&gt;='Methodology'!$G$10,'Methodology'!$H$10,'Methodology'!$H$11)))))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -9871,7 +10251,7 @@
       </x:c>
       <x:c r="D12" s="17" t="n">
         <x:f>COUNTIF('Observations'!$A$6:$A$500,A12)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
         <x:f>IF(D12&lt;3,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A12,'Observations'!$F$6:$F$500,"&lt;"&amp;F12))</x:f>
@@ -9879,8 +10259,9 @@
       <x:c r="F12" s="17" t="str">
         <x:f>IF(D12&lt;2,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A12,'Observations'!$F$6:$F$500,"&lt;"&amp;G12))</x:f>
       </x:c>
-      <x:c r="G12" s="17" t="str">
+      <x:c r="G12" s="17" t="n">
         <x:f>IF(D12=0,"",MAXIFS('Observations'!$F$6:$F$500,'Observations'!$A$6:$A$500,A12))</x:f>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
         <x:f>IF(E12="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A12,'Observations'!$F$6:$F$500,E12))</x:f>
@@ -9888,17 +10269,19 @@
       <x:c r="I12" s="24" t="str">
         <x:f>IF(F12="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A12,'Observations'!$F$6:$F$500,F12))</x:f>
       </x:c>
-      <x:c r="J12" s="24" t="str">
+      <x:c r="J12" s="24" t="n">
         <x:f>IF(G12="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A12,'Observations'!$F$6:$F$500,G12))</x:f>
+        <x:v>0.273</x:v>
       </x:c>
       <x:c r="K12" s="25" t="str">
-        <x:f>IF(H12="","",-LN(1-H12)/LN(2))</x:f>
+        <x:f>IF(H12="","",IF(H12&gt;=1,30,-LN(1-H12)/LN(2)))</x:f>
       </x:c>
       <x:c r="L12" s="25" t="str">
-        <x:f>IF(I12="","",-LN(1-I12)/LN(2))</x:f>
-      </x:c>
-      <x:c r="M12" s="25" t="str">
-        <x:f>IF(J12="","",-LN(1-J12)/LN(2))</x:f>
+        <x:f>IF(I12="","",IF(I12&gt;=1,30,-LN(1-I12)/LN(2)))</x:f>
+      </x:c>
+      <x:c r="M12" s="25" t="n">
+        <x:f>IF(J12="","",IF(J12&gt;=1,30,-LN(1-J12)/LN(2)))</x:f>
+        <x:v>0.45997273074249273</x:v>
       </x:c>
       <x:c r="N12" s="25" t="n">
         <x:f>IF(D12&lt;2,0,(M12-L12)/(G12-F12))</x:f>
@@ -9914,17 +10297,19 @@
       </x:c>
       <x:c r="Q12" s="17" t="str">
         <x:f>IF(D12=0,"Ungraded — no normalized observation",IF(D12=1,"Flat — one observation",IF(D12=2,"Constant velocity — two observations","Velocity + acceleration — latest three observations")))</x:f>
-        <x:v>Ungraded — no normalized observation</x:v>
-      </x:c>
-      <x:c r="R12" s="24" t="str">
+        <x:v>Flat — one observation</x:v>
+      </x:c>
+      <x:c r="R12" s="24" t="n">
         <x:f>IF(D12=0,"",J12)</x:f>
+        <x:v>0.273</x:v>
       </x:c>
       <x:c r="S12" s="17" t="str">
         <x:f>IF(R12="","N/A",IF(R12&gt;='Methodology'!$G$7,"A",IF(R12&gt;='Methodology'!$G$8,"B",IF(R12&gt;='Methodology'!$G$9,"C",IF(R12&gt;='Methodology'!$G$10,"D","F")))))</x:f>
-        <x:v>N/A</x:v>
-      </x:c>
-      <x:c r="T12" s="26" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="T12" s="26" t="n">
         <x:f>IF(R12="","",IF(R12&gt;='Methodology'!$G$7,'Methodology'!$H$7,IF(R12&gt;='Methodology'!$G$8,'Methodology'!$H$8,IF(R12&gt;='Methodology'!$G$9,'Methodology'!$H$9,IF(R12&gt;='Methodology'!$G$10,'Methodology'!$H$10,'Methodology'!$H$11)))))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -9964,14 +10349,14 @@
         <x:v>0.503</x:v>
       </x:c>
       <x:c r="K13" s="25" t="str">
-        <x:f>IF(H13="","",-LN(1-H13)/LN(2))</x:f>
+        <x:f>IF(H13="","",IF(H13&gt;=1,30,-LN(1-H13)/LN(2)))</x:f>
       </x:c>
       <x:c r="L13" s="25" t="n">
-        <x:f>IF(I13="","",-LN(1-I13)/LN(2))</x:f>
+        <x:f>IF(I13="","",IF(I13&gt;=1,30,-LN(1-I13)/LN(2)))</x:f>
         <x:v>0.8935176695300188</x:v>
       </x:c>
       <x:c r="M13" s="25" t="n">
-        <x:f>IF(J13="","",-LN(1-J13)/LN(2))</x:f>
+        <x:f>IF(J13="","",IF(J13&gt;=1,30,-LN(1-J13)/LN(2)))</x:f>
         <x:v>1.008682243099801</x:v>
       </x:c>
       <x:c r="N13" s="25" t="n">
@@ -10042,15 +10427,15 @@
         <x:v>0.511</x:v>
       </x:c>
       <x:c r="K14" s="25" t="n">
-        <x:f>IF(H14="","",-LN(1-H14)/LN(2))</x:f>
+        <x:f>IF(H14="","",IF(H14&gt;=1,30,-LN(1-H14)/LN(2)))</x:f>
         <x:v>0.7226103011891362</x:v>
       </x:c>
       <x:c r="L14" s="25" t="n">
-        <x:f>IF(I14="","",-LN(1-I14)/LN(2))</x:f>
+        <x:f>IF(I14="","",IF(I14&gt;=1,30,-LN(1-I14)/LN(2)))</x:f>
         <x:v>0.8862995008352721</x:v>
       </x:c>
       <x:c r="M14" s="25" t="n">
-        <x:f>IF(J14="","",-LN(1-J14)/LN(2))</x:f>
+        <x:f>IF(J14="","",IF(J14&gt;=1,30,-LN(1-J14)/LN(2)))</x:f>
         <x:v>1.0320936297098533</x:v>
       </x:c>
       <x:c r="N14" s="25" t="n">
@@ -10121,15 +10506,15 @@
         <x:v>0.607</x:v>
       </x:c>
       <x:c r="K15" s="25" t="n">
-        <x:f>IF(H15="","",-LN(1-H15)/LN(2))</x:f>
+        <x:f>IF(H15="","",IF(H15&gt;=1,30,-LN(1-H15)/LN(2)))</x:f>
         <x:v>0.49410907027004275</x:v>
       </x:c>
       <x:c r="L15" s="25" t="n">
-        <x:f>IF(I15="","",-LN(1-I15)/LN(2))</x:f>
+        <x:f>IF(I15="","",IF(I15&gt;=1,30,-LN(1-I15)/LN(2)))</x:f>
         <x:v>1.0679388286565756</x:v>
       </x:c>
       <x:c r="M15" s="25" t="n">
-        <x:f>IF(J15="","",-LN(1-J15)/LN(2))</x:f>
+        <x:f>IF(J15="","",IF(J15&gt;=1,30,-LN(1-J15)/LN(2)))</x:f>
         <x:v>1.3473987824034805</x:v>
       </x:c>
       <x:c r="N15" s="25" t="n">
@@ -10196,13 +10581,13 @@
         <x:v>0.758</x:v>
       </x:c>
       <x:c r="K16" s="25" t="str">
-        <x:f>IF(H16="","",-LN(1-H16)/LN(2))</x:f>
+        <x:f>IF(H16="","",IF(H16&gt;=1,30,-LN(1-H16)/LN(2)))</x:f>
       </x:c>
       <x:c r="L16" s="25" t="str">
-        <x:f>IF(I16="","",-LN(1-I16)/LN(2))</x:f>
+        <x:f>IF(I16="","",IF(I16&gt;=1,30,-LN(1-I16)/LN(2)))</x:f>
       </x:c>
       <x:c r="M16" s="25" t="n">
-        <x:f>IF(J16="","",-LN(1-J16)/LN(2))</x:f>
+        <x:f>IF(J16="","",IF(J16&gt;=1,30,-LN(1-J16)/LN(2)))</x:f>
         <x:v>2.046921047387493</x:v>
       </x:c>
       <x:c r="N16" s="25" t="n">
@@ -10273,15 +10658,15 @@
         <x:v>0.429</x:v>
       </x:c>
       <x:c r="K17" s="25" t="n">
-        <x:f>IF(H17="","",-LN(1-H17)/LN(2))</x:f>
+        <x:f>IF(H17="","",IF(H17&gt;=1,30,-LN(1-H17)/LN(2)))</x:f>
         <x:v>0.3959286763311392</x:v>
       </x:c>
       <x:c r="L17" s="25" t="n">
-        <x:f>IF(I17="","",-LN(1-I17)/LN(2))</x:f>
+        <x:f>IF(I17="","",IF(I17&gt;=1,30,-LN(1-I17)/LN(2)))</x:f>
         <x:v>0.5207694387936639</x:v>
       </x:c>
       <x:c r="M17" s="25" t="n">
-        <x:f>IF(J17="","",-LN(1-J17)/LN(2))</x:f>
+        <x:f>IF(J17="","",IF(J17&gt;=1,30,-LN(1-J17)/LN(2)))</x:f>
         <x:v>0.8084373492992445</x:v>
       </x:c>
       <x:c r="N17" s="25" t="n">
@@ -10346,13 +10731,13 @@
         <x:f>IF(G18="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A18,'Observations'!$F$6:$F$500,G18))</x:f>
       </x:c>
       <x:c r="K18" s="25" t="str">
-        <x:f>IF(H18="","",-LN(1-H18)/LN(2))</x:f>
+        <x:f>IF(H18="","",IF(H18&gt;=1,30,-LN(1-H18)/LN(2)))</x:f>
       </x:c>
       <x:c r="L18" s="25" t="str">
-        <x:f>IF(I18="","",-LN(1-I18)/LN(2))</x:f>
+        <x:f>IF(I18="","",IF(I18&gt;=1,30,-LN(1-I18)/LN(2)))</x:f>
       </x:c>
       <x:c r="M18" s="25" t="str">
-        <x:f>IF(J18="","",-LN(1-J18)/LN(2))</x:f>
+        <x:f>IF(J18="","",IF(J18&gt;=1,30,-LN(1-J18)/LN(2)))</x:f>
       </x:c>
       <x:c r="N18" s="25" t="n">
         <x:f>IF(D18&lt;2,0,(M18-L18)/(G18-F18))</x:f>
@@ -10416,13 +10801,13 @@
         <x:v>0.384</x:v>
       </x:c>
       <x:c r="K19" s="25" t="str">
-        <x:f>IF(H19="","",-LN(1-H19)/LN(2))</x:f>
+        <x:f>IF(H19="","",IF(H19&gt;=1,30,-LN(1-H19)/LN(2)))</x:f>
       </x:c>
       <x:c r="L19" s="25" t="str">
-        <x:f>IF(I19="","",-LN(1-I19)/LN(2))</x:f>
+        <x:f>IF(I19="","",IF(I19&gt;=1,30,-LN(1-I19)/LN(2)))</x:f>
       </x:c>
       <x:c r="M19" s="25" t="n">
-        <x:f>IF(J19="","",-LN(1-J19)/LN(2))</x:f>
+        <x:f>IF(J19="","",IF(J19&gt;=1,30,-LN(1-J19)/LN(2)))</x:f>
         <x:v>0.6989977439671857</x:v>
       </x:c>
       <x:c r="N19" s="25" t="n">
@@ -10493,15 +10878,15 @@
         <x:v>0.552</x:v>
       </x:c>
       <x:c r="K20" s="25" t="n">
-        <x:f>IF(H20="","",-LN(1-H20)/LN(2))</x:f>
+        <x:f>IF(H20="","",IF(H20&gt;=1,30,-LN(1-H20)/LN(2)))</x:f>
         <x:v>0.7226103011891362</x:v>
       </x:c>
       <x:c r="L20" s="25" t="n">
-        <x:f>IF(I20="","",-LN(1-I20)/LN(2))</x:f>
+        <x:f>IF(I20="","",IF(I20&gt;=1,30,-LN(1-I20)/LN(2)))</x:f>
         <x:v>0.8520421186128986</x:v>
       </x:c>
       <x:c r="M20" s="25" t="n">
-        <x:f>IF(J20="","",-LN(1-J20)/LN(2))</x:f>
+        <x:f>IF(J20="","",IF(J20&gt;=1,30,-LN(1-J20)/LN(2)))</x:f>
         <x:v>1.158429362604483</x:v>
       </x:c>
       <x:c r="N20" s="25" t="n">
@@ -10568,13 +10953,13 @@
         <x:v>0.582</x:v>
       </x:c>
       <x:c r="K21" s="25" t="str">
-        <x:f>IF(H21="","",-LN(1-H21)/LN(2))</x:f>
+        <x:f>IF(H21="","",IF(H21&gt;=1,30,-LN(1-H21)/LN(2)))</x:f>
       </x:c>
       <x:c r="L21" s="25" t="str">
-        <x:f>IF(I21="","",-LN(1-I21)/LN(2))</x:f>
+        <x:f>IF(I21="","",IF(I21&gt;=1,30,-LN(1-I21)/LN(2)))</x:f>
       </x:c>
       <x:c r="M21" s="25" t="n">
-        <x:f>IF(J21="","",-LN(1-J21)/LN(2))</x:f>
+        <x:f>IF(J21="","",IF(J21&gt;=1,30,-LN(1-J21)/LN(2)))</x:f>
         <x:v>1.2584251525812042</x:v>
       </x:c>
       <x:c r="N21" s="25" t="n">
@@ -10641,13 +11026,13 @@
         <x:v>0.676</x:v>
       </x:c>
       <x:c r="K22" s="25" t="str">
-        <x:f>IF(H22="","",-LN(1-H22)/LN(2))</x:f>
+        <x:f>IF(H22="","",IF(H22&gt;=1,30,-LN(1-H22)/LN(2)))</x:f>
       </x:c>
       <x:c r="L22" s="25" t="str">
-        <x:f>IF(I22="","",-LN(1-I22)/LN(2))</x:f>
+        <x:f>IF(I22="","",IF(I22&gt;=1,30,-LN(1-I22)/LN(2)))</x:f>
       </x:c>
       <x:c r="M22" s="25" t="n">
-        <x:f>IF(J22="","",-LN(1-J22)/LN(2))</x:f>
+        <x:f>IF(J22="","",IF(J22&gt;=1,30,-LN(1-J22)/LN(2)))</x:f>
         <x:v>1.6259342817774625</x:v>
       </x:c>
       <x:c r="N22" s="25" t="n">
@@ -10714,13 +11099,13 @@
         <x:v>0.333</x:v>
       </x:c>
       <x:c r="K23" s="25" t="str">
-        <x:f>IF(H23="","",-LN(1-H23)/LN(2))</x:f>
+        <x:f>IF(H23="","",IF(H23&gt;=1,30,-LN(1-H23)/LN(2)))</x:f>
       </x:c>
       <x:c r="L23" s="25" t="str">
-        <x:f>IF(I23="","",-LN(1-I23)/LN(2))</x:f>
+        <x:f>IF(I23="","",IF(I23&gt;=1,30,-LN(1-I23)/LN(2)))</x:f>
       </x:c>
       <x:c r="M23" s="25" t="n">
-        <x:f>IF(J23="","",-LN(1-J23)/LN(2))</x:f>
+        <x:f>IF(J23="","",IF(J23&gt;=1,30,-LN(1-J23)/LN(2)))</x:f>
         <x:v>0.584241333477502</x:v>
       </x:c>
       <x:c r="N23" s="25" t="n">
@@ -10789,14 +11174,14 @@
         <x:v>0.367</x:v>
       </x:c>
       <x:c r="K24" s="25" t="str">
-        <x:f>IF(H24="","",-LN(1-H24)/LN(2))</x:f>
+        <x:f>IF(H24="","",IF(H24&gt;=1,30,-LN(1-H24)/LN(2)))</x:f>
       </x:c>
       <x:c r="L24" s="25" t="n">
-        <x:f>IF(I24="","",-LN(1-I24)/LN(2))</x:f>
+        <x:f>IF(I24="","",IF(I24&gt;=1,30,-LN(1-I24)/LN(2)))</x:f>
         <x:v>0.41888982477445036</x:v>
       </x:c>
       <x:c r="M24" s="25" t="n">
-        <x:f>IF(J24="","",-LN(1-J24)/LN(2))</x:f>
+        <x:f>IF(J24="","",IF(J24&gt;=1,30,-LN(1-J24)/LN(2)))</x:f>
         <x:v>0.6597225952337457</x:v>
       </x:c>
       <x:c r="N24" s="25" t="n">
@@ -10861,13 +11246,13 @@
         <x:f>IF(G25="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A25,'Observations'!$F$6:$F$500,G25))</x:f>
       </x:c>
       <x:c r="K25" s="25" t="str">
-        <x:f>IF(H25="","",-LN(1-H25)/LN(2))</x:f>
+        <x:f>IF(H25="","",IF(H25&gt;=1,30,-LN(1-H25)/LN(2)))</x:f>
       </x:c>
       <x:c r="L25" s="25" t="str">
-        <x:f>IF(I25="","",-LN(1-I25)/LN(2))</x:f>
+        <x:f>IF(I25="","",IF(I25&gt;=1,30,-LN(1-I25)/LN(2)))</x:f>
       </x:c>
       <x:c r="M25" s="25" t="str">
-        <x:f>IF(J25="","",-LN(1-J25)/LN(2))</x:f>
+        <x:f>IF(J25="","",IF(J25&gt;=1,30,-LN(1-J25)/LN(2)))</x:f>
       </x:c>
       <x:c r="N25" s="25" t="n">
         <x:f>IF(D25&lt;2,0,(M25-L25)/(G25-F25))</x:f>
@@ -10935,15 +11320,15 @@
         <x:v>0.158</x:v>
       </x:c>
       <x:c r="K26" s="25" t="n">
-        <x:f>IF(H26="","",-LN(1-H26)/LN(2))</x:f>
+        <x:f>IF(H26="","",IF(H26&gt;=1,30,-LN(1-H26)/LN(2)))</x:f>
         <x:v>0.05514155419246095</x:v>
       </x:c>
       <x:c r="L26" s="25" t="n">
-        <x:f>IF(I26="","",-LN(1-I26)/LN(2))</x:f>
+        <x:f>IF(I26="","",IF(I26&gt;=1,30,-LN(1-I26)/LN(2)))</x:f>
         <x:v>0.06145072623394566</x:v>
       </x:c>
       <x:c r="M26" s="25" t="n">
-        <x:f>IF(J26="","",-LN(1-J26)/LN(2))</x:f>
+        <x:f>IF(J26="","",IF(J26&gt;=1,30,-LN(1-J26)/LN(2)))</x:f>
         <x:v>0.24810786159569104</x:v>
       </x:c>
       <x:c r="N26" s="25" t="n">
@@ -11008,13 +11393,13 @@
         <x:f>IF(G27="","",SUMIFS('Observations'!$G$6:$G$500,'Observations'!$A$6:$A$500,A27,'Observations'!$F$6:$F$500,G27))</x:f>
       </x:c>
       <x:c r="K27" s="25" t="str">
-        <x:f>IF(H27="","",-LN(1-H27)/LN(2))</x:f>
+        <x:f>IF(H27="","",IF(H27&gt;=1,30,-LN(1-H27)/LN(2)))</x:f>
       </x:c>
       <x:c r="L27" s="25" t="str">
-        <x:f>IF(I27="","",-LN(1-I27)/LN(2))</x:f>
+        <x:f>IF(I27="","",IF(I27&gt;=1,30,-LN(1-I27)/LN(2)))</x:f>
       </x:c>
       <x:c r="M27" s="25" t="str">
-        <x:f>IF(J27="","",-LN(1-J27)/LN(2))</x:f>
+        <x:f>IF(J27="","",IF(J27&gt;=1,30,-LN(1-J27)/LN(2)))</x:f>
       </x:c>
       <x:c r="N27" s="25" t="n">
         <x:f>IF(D27&lt;2,0,(M27-L27)/(G27-F27))</x:f>
@@ -11078,13 +11463,13 @@
         <x:v>0.704</x:v>
       </x:c>
       <x:c r="K28" s="25" t="str">
-        <x:f>IF(H28="","",-LN(1-H28)/LN(2))</x:f>
+        <x:f>IF(H28="","",IF(H28&gt;=1,30,-LN(1-H28)/LN(2)))</x:f>
       </x:c>
       <x:c r="L28" s="25" t="str">
-        <x:f>IF(I28="","",-LN(1-I28)/LN(2))</x:f>
+        <x:f>IF(I28="","",IF(I28&gt;=1,30,-LN(1-I28)/LN(2)))</x:f>
       </x:c>
       <x:c r="M28" s="25" t="n">
-        <x:f>IF(J28="","",-LN(1-J28)/LN(2))</x:f>
+        <x:f>IF(J28="","",IF(J28&gt;=1,30,-LN(1-J28)/LN(2)))</x:f>
         <x:v>1.756330919033137</x:v>
       </x:c>
       <x:c r="N28" s="25" t="n">
@@ -11123,7 +11508,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R559f98929afb46ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f0578419a2f4262"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11430,7 +11815,20 @@
         <x:v>No score is fabricated before release or without a normalized observation</x:v>
       </x:c>
     </x:row>
-    <x:row r="14"/>
+    <x:row r="14" ht="21.600000381469727" hidden="0" customHeight="1">
+      <x:c r="A14" s="17" t="str">
+        <x:v>Acceleration summary</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>Observed series only</x:v>
+      </x:c>
+      <x:c r="C14" s="17" t="str">
+        <x:v>rule</x:v>
+      </x:c>
+      <x:c r="D14" s="17" t="str">
+        <x:v>Average 3+ point acceleration estimates; coverage is reported separately</x:v>
+      </x:c>
+    </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="9" t="str">
         <x:v>FORECAST EQUATIONS AND INTERPRETATION</x:v>
@@ -11489,7 +11887,7 @@
         <x:v>d = -LOG2(1 - score)</x:v>
       </x:c>
       <x:c r="C17" s="17" t="str">
-        <x:v>Transforms a bounded percentage into halvings of the remaining failure gap.</x:v>
+        <x:v>Transforms a bounded percentage into halvings of the remaining failure gap. Exact 100% is represented as 30 halvings for finite computation.</x:v>
       </x:c>
       <x:c r="D17" s="17"/>
       <x:c r="E17" s="17"/>
@@ -11507,7 +11905,7 @@
         <x:v>v = (d_t - d_t-1) / elapsed quarters</x:v>
       </x:c>
       <x:c r="C18" s="17" t="str">
-        <x:v>First derivative of failure-gap depth. Report-card Rate cells separately show score percentage-point changes.</x:v>
+        <x:v>First derivative of failure-gap depth. Report-card Δ score cells separately show quarter-over-quarter percentage-point changes.</x:v>
       </x:c>
       <x:c r="D18" s="17"/>
       <x:c r="E18" s="17"/>
@@ -11592,42 +11990,42 @@
     <x:row r="23"/>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="F24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="I24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
+        <x:v>NORMALIZATION RULES</x:v>
       </x:c>
       <x:c r="J24" s="9" t="str">
-        <x:v>COMPOSITE RULES</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="34" hidden="0" customHeight="1">
+        <x:v>NORMALIZATION RULES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="38" hidden="0" customHeight="1">
       <x:c r="A25" s="13" t="str">
-        <x:v>Rule</x:v>
+        <x:v>Metric type</x:v>
       </x:c>
       <x:c r="B25" s="13" t="str">
-        <x:v>Definition</x:v>
+        <x:v>Conversion to 0–100%</x:v>
       </x:c>
       <x:c r="C25" s="13"/>
       <x:c r="D25" s="13"/>
@@ -11638,12 +12036,12 @@
       <x:c r="I25" s="13"/>
       <x:c r="J25" s="13"/>
     </x:row>
-    <x:row r="26" ht="34" hidden="0" customHeight="1">
+    <x:row r="26" ht="38" hidden="0" customHeight="1">
       <x:c r="A26" s="17" t="str">
-        <x:v>Current benchmark grade</x:v>
+        <x:v>Native percentage</x:v>
       </x:c>
       <x:c r="B26" s="17" t="str">
-        <x:v>Latest observed frontier carried to 2026-Q3; A ≥90%, B ≥80%, C ≥70%, D ≥60%, F &lt;60%.</x:v>
+        <x:v>Use the strict pass, completion, survival, or rubric score as published; pin the benchmark and evaluation configuration.</x:v>
       </x:c>
       <x:c r="C26" s="17"/>
       <x:c r="D26" s="17"/>
@@ -11654,12 +12052,12 @@
       <x:c r="I26" s="17"/>
       <x:c r="J26" s="17"/>
     </x:row>
-    <x:row r="27" ht="34" hidden="0" customHeight="1">
+    <x:row r="27" ht="38" hidden="0" customHeight="1">
       <x:c r="A27" s="17" t="str">
-        <x:v>Benchmark GPA</x:v>
+        <x:v>Terminal money</x:v>
       </x:c>
       <x:c r="B27" s="17" t="str">
-        <x:v>A=4, B=3, C=2, D=1, F=0. Ungraded benchmarks are excluded, not assigned zero.</x:v>
+        <x:v>Frontier terminal outcome ÷ a fixed published target, human result, expert strategy, or oracle result; cap at 100%.</x:v>
       </x:c>
       <x:c r="C27" s="17"/>
       <x:c r="D27" s="17"/>
@@ -11670,12 +12068,12 @@
       <x:c r="I27" s="17"/>
       <x:c r="J27" s="17"/>
     </x:row>
-    <x:row r="28" ht="34" hidden="0" customHeight="1">
+    <x:row r="28" ht="38" hidden="0" customHeight="1">
       <x:c r="A28" s="17" t="str">
-        <x:v>Category GPA</x:v>
+        <x:v>Target-only money</x:v>
       </x:c>
       <x:c r="B28" s="17" t="str">
-        <x:v>Mean GPA of graded benchmarks within the category.</x:v>
+        <x:v>If no human/oracle result exists, a source-published success target may be used provisionally and must be labeled when saturated.</x:v>
       </x:c>
       <x:c r="C28" s="17"/>
       <x:c r="D28" s="17"/>
@@ -11686,12 +12084,12 @@
       <x:c r="I28" s="17"/>
       <x:c r="J28" s="17"/>
     </x:row>
-    <x:row r="29" ht="34" hidden="0" customHeight="1">
+    <x:row r="29" ht="38" hidden="0" customHeight="1">
       <x:c r="A29" s="17" t="str">
-        <x:v>Overall GPA</x:v>
+        <x:v>Elo</x:v>
       </x:c>
       <x:c r="B29" s="17" t="str">
-        <x:v>Mean of the four category GPAs. Equal category weighting prevents categories with more benchmarks from dominating.</x:v>
+        <x:v>Convert to win probability against a fixed named anchor: p = 1 / (1 + 10^((R_anchor − R_system)/400)). Never min–max a changing leaderboard.</x:v>
       </x:c>
       <x:c r="C29" s="17"/>
       <x:c r="D29" s="17"/>
@@ -11702,12 +12100,12 @@
       <x:c r="I29" s="17"/>
       <x:c r="J29" s="17"/>
     </x:row>
-    <x:row r="30" ht="34" hidden="0" customHeight="1">
+    <x:row r="30" ht="38" hidden="0" customHeight="1">
       <x:c r="A30" s="17" t="str">
-        <x:v>Overall score</x:v>
+        <x:v>Guardrail</x:v>
       </x:c>
       <x:c r="B30" s="17" t="str">
-        <x:v>Mean of the four category mean scores after all benchmark metrics have been normalized to 0–100% completion/saturation.</x:v>
+        <x:v>Do not mix ratios to different anchors in one series. A changed task, harness, judge, budget, or anchor is a documented series break.</x:v>
       </x:c>
       <x:c r="C30" s="17"/>
       <x:c r="D30" s="17"/>
@@ -11721,58 +12119,58 @@
     <x:row r="31"/>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="B32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="H32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
       <x:c r="J32" s="9" t="str">
-        <x:v>UPDATE PROTOCOL</x:v>
+        <x:v>COMPOSITE RULES</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" hidden="0" customHeight="1">
-      <x:c r="A33" s="23" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B33" s="17" t="str">
-        <x:v>Append one row to Observations for each new comparable benchmark result; keep benchmark ID and quarter index intact.</x:v>
-      </x:c>
-      <x:c r="C33" s="17"/>
-      <x:c r="D33" s="17"/>
-      <x:c r="E33" s="17"/>
-      <x:c r="F33" s="17"/>
-      <x:c r="G33" s="17"/>
-      <x:c r="H33" s="17"/>
-      <x:c r="I33" s="17"/>
-      <x:c r="J33" s="17"/>
+      <x:c r="A33" s="13" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B33" s="13" t="str">
+        <x:v>Definition</x:v>
+      </x:c>
+      <x:c r="C33" s="13"/>
+      <x:c r="D33" s="13"/>
+      <x:c r="E33" s="13"/>
+      <x:c r="F33" s="13"/>
+      <x:c r="G33" s="13"/>
+      <x:c r="H33" s="13"/>
+      <x:c r="I33" s="13"/>
+      <x:c r="J33" s="13"/>
     </x:row>
     <x:row r="34" ht="34" hidden="0" customHeight="1">
-      <x:c r="A34" s="23" t="str">
-        <x:v>2</x:v>
+      <x:c r="A34" s="17" t="str">
+        <x:v>Current benchmark grade</x:v>
       </x:c>
       <x:c r="B34" s="17" t="str">
-        <x:v>Use the release quarter, not the date the analyst happened to discover the result. Keep only the quarter frontier for a fixed benchmark/harness definition.</x:v>
+        <x:v>Latest observed frontier carried to 2026-Q3; A ≥90%, B ≥80%, C ≥70%, D ≥60%, F &lt;60%.</x:v>
       </x:c>
       <x:c r="C34" s="17"/>
       <x:c r="D34" s="17"/>
@@ -11784,11 +12182,11 @@
       <x:c r="J34" s="17"/>
     </x:row>
     <x:row r="35" ht="34" hidden="0" customHeight="1">
-      <x:c r="A35" s="23" t="str">
-        <x:v>3</x:v>
+      <x:c r="A35" s="17" t="str">
+        <x:v>Benchmark GPA</x:v>
       </x:c>
       <x:c r="B35" s="17" t="str">
-        <x:v>If the task set, harness, judge, retry policy, tools, or budget changes, describe the break in Notes and decide whether the row belongs in the same series.</x:v>
+        <x:v>A=4, B=3, C=2, D=1, F=0. Ungraded benchmarks are excluded, not assigned zero.</x:v>
       </x:c>
       <x:c r="C35" s="17"/>
       <x:c r="D35" s="17"/>
@@ -11800,11 +12198,11 @@
       <x:c r="J35" s="17"/>
     </x:row>
     <x:row r="36" ht="34" hidden="0" customHeight="1">
-      <x:c r="A36" s="23" t="str">
-        <x:v>4</x:v>
+      <x:c r="A36" s="17" t="str">
+        <x:v>Category GPA</x:v>
       </x:c>
       <x:c r="B36" s="17" t="str">
-        <x:v>Add new benchmarks to Catalog and Report Card only when their metric can be normalized without an arbitrary denominator.</x:v>
+        <x:v>Mean GPA of graded benchmarks within the category.</x:v>
       </x:c>
       <x:c r="C36" s="17"/>
       <x:c r="D36" s="17"/>
@@ -11816,11 +12214,11 @@
       <x:c r="J36" s="17"/>
     </x:row>
     <x:row r="37" ht="34" hidden="0" customHeight="1">
-      <x:c r="A37" s="23" t="str">
-        <x:v>5</x:v>
+      <x:c r="A37" s="17" t="str">
+        <x:v>Overall GPA</x:v>
       </x:c>
       <x:c r="B37" s="17" t="str">
-        <x:v>Refresh sources and inspect projected saturation. A projection is a scenario extrapolation, not a probability distribution.</x:v>
+        <x:v>Mean of the four category GPAs. Equal category weighting prevents categories with more benchmarks from dominating.</x:v>
       </x:c>
       <x:c r="C37" s="17"/>
       <x:c r="D37" s="17"/>
@@ -11830,6 +12228,135 @@
       <x:c r="H37" s="17"/>
       <x:c r="I37" s="17"/>
       <x:c r="J37" s="17"/>
+    </x:row>
+    <x:row r="38" ht="34" hidden="0" customHeight="1">
+      <x:c r="A38" s="17" t="str">
+        <x:v>Overall score</x:v>
+      </x:c>
+      <x:c r="B38" s="17" t="str">
+        <x:v>Mean of the four category mean scores after all benchmark metrics have been normalized to 0–100% completion/saturation.</x:v>
+      </x:c>
+      <x:c r="C38" s="17"/>
+      <x:c r="D38" s="17"/>
+      <x:c r="E38" s="17"/>
+      <x:c r="F38" s="17"/>
+      <x:c r="G38" s="17"/>
+      <x:c r="H38" s="17"/>
+      <x:c r="I38" s="17"/>
+      <x:c r="J38" s="17"/>
+    </x:row>
+    <x:row r="39"/>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="B40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="C40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="D40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="E40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="G40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="H40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="I40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+      <x:c r="J40" s="9" t="str">
+        <x:v>UPDATE PROTOCOL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="34" hidden="0" customHeight="1">
+      <x:c r="A41" s="23" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B41" s="17" t="str">
+        <x:v>Append one row to Observations for each new comparable benchmark result; keep benchmark ID and quarter index intact.</x:v>
+      </x:c>
+      <x:c r="C41" s="17"/>
+      <x:c r="D41" s="17"/>
+      <x:c r="E41" s="17"/>
+      <x:c r="F41" s="17"/>
+      <x:c r="G41" s="17"/>
+      <x:c r="H41" s="17"/>
+      <x:c r="I41" s="17"/>
+      <x:c r="J41" s="17"/>
+    </x:row>
+    <x:row r="42" ht="34" hidden="0" customHeight="1">
+      <x:c r="A42" s="23" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B42" s="17" t="str">
+        <x:v>Use the release quarter, not the date the analyst happened to discover the result. Keep only the quarter frontier for a fixed benchmark/harness definition.</x:v>
+      </x:c>
+      <x:c r="C42" s="17"/>
+      <x:c r="D42" s="17"/>
+      <x:c r="E42" s="17"/>
+      <x:c r="F42" s="17"/>
+      <x:c r="G42" s="17"/>
+      <x:c r="H42" s="17"/>
+      <x:c r="I42" s="17"/>
+      <x:c r="J42" s="17"/>
+    </x:row>
+    <x:row r="43" ht="34" hidden="0" customHeight="1">
+      <x:c r="A43" s="23" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B43" s="17" t="str">
+        <x:v>If the task set, harness, judge, retry policy, tools, or budget changes, describe the break in Notes and decide whether the row belongs in the same series.</x:v>
+      </x:c>
+      <x:c r="C43" s="17"/>
+      <x:c r="D43" s="17"/>
+      <x:c r="E43" s="17"/>
+      <x:c r="F43" s="17"/>
+      <x:c r="G43" s="17"/>
+      <x:c r="H43" s="17"/>
+      <x:c r="I43" s="17"/>
+      <x:c r="J43" s="17"/>
+    </x:row>
+    <x:row r="44" ht="34" hidden="0" customHeight="1">
+      <x:c r="A44" s="23" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B44" s="17" t="str">
+        <x:v>Add new benchmarks to Catalog and Report Card only when their metric can be normalized without an arbitrary denominator.</x:v>
+      </x:c>
+      <x:c r="C44" s="17"/>
+      <x:c r="D44" s="17"/>
+      <x:c r="E44" s="17"/>
+      <x:c r="F44" s="17"/>
+      <x:c r="G44" s="17"/>
+      <x:c r="H44" s="17"/>
+      <x:c r="I44" s="17"/>
+      <x:c r="J44" s="17"/>
+    </x:row>
+    <x:row r="45" ht="34" hidden="0" customHeight="1">
+      <x:c r="A45" s="23" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B45" s="17" t="str">
+        <x:v>Refresh sources and inspect projected saturation. A projection is a scenario extrapolation, not a probability distribution.</x:v>
+      </x:c>
+      <x:c r="C45" s="17"/>
+      <x:c r="D45" s="17"/>
+      <x:c r="E45" s="17"/>
+      <x:c r="F45" s="17"/>
+      <x:c r="G45" s="17"/>
+      <x:c r="H45" s="17"/>
+      <x:c r="I45" s="17"/>
+      <x:c r="J45" s="17"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -11858,6 +12385,13 @@
     <x:mergeCell ref="B35:J35"/>
     <x:mergeCell ref="B36:J36"/>
     <x:mergeCell ref="B37:J37"/>
+    <x:mergeCell ref="B38:J38"/>
+    <x:mergeCell ref="A40:J40"/>
+    <x:mergeCell ref="B41:J41"/>
+    <x:mergeCell ref="B42:J42"/>
+    <x:mergeCell ref="B43:J43"/>
+    <x:mergeCell ref="B44:J44"/>
+    <x:mergeCell ref="B45:J45"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>